<commit_message>
atualização banco de dados
</commit_message>
<xml_diff>
--- a/tratando_tabelas/finitura/entradas_finitura.xlsx
+++ b/tratando_tabelas/finitura/entradas_finitura.xlsx
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1112" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1072" uniqueCount="195">
   <si>
     <t xml:space="preserve">Santri ADM 1.1.5.7 R1</t>
   </si>
   <si>
-    <t xml:space="preserve">Emitido em: 18/05/2026 07:30:58</t>
+    <t xml:space="preserve">Emitido em: 19/05/2026 05:30:31</t>
   </si>
   <si>
     <t xml:space="preserve">Relação de entradas - Sintético</t>
@@ -265,28 +265,13 @@
     <t xml:space="preserve">Não</t>
   </si>
   <si>
-    <t xml:space="preserve">547 - LORENZETTI S/A INDU.BRASILEIRAS ELETROMETALURGICAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.972.380</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30/04/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.384,20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.910</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35260461413282000143550010029723801722131595</t>
-  </si>
-  <si>
     <t xml:space="preserve">30.850 - DEXCO S.A</t>
   </si>
   <si>
     <t xml:space="preserve">161.164</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30/04/2026</t>
   </si>
   <si>
     <t xml:space="preserve">05/05/2026</t>
@@ -331,10 +316,19 @@
     <t xml:space="preserve">43260586895448000136550010000648961248387979</t>
   </si>
   <si>
-    <t xml:space="preserve">64.895</t>
+    <t xml:space="preserve">64.894</t>
   </si>
   <si>
     <t xml:space="preserve">07/05/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.725,01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">43260586895448000136550010000648941804845676</t>
+  </si>
+  <si>
+    <t xml:space="preserve">64.895</t>
   </si>
   <si>
     <t xml:space="preserve">1.978,02</t>
@@ -347,6 +341,9 @@
   </si>
   <si>
     <t xml:space="preserve">569,02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.910</t>
   </si>
   <si>
     <t xml:space="preserve">43260586895448000136550010000648971591022939</t>
@@ -403,25 +400,10 @@
     <t xml:space="preserve">35260512077181000133550030002245691053712641</t>
   </si>
   <si>
-    <t xml:space="preserve">26.619 - DICAN COMERCIO EXTERIOR LTDA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">120.077</t>
+    <t xml:space="preserve">64.914</t>
   </si>
   <si>
     <t xml:space="preserve">08/05/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05/06/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.625,80</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35260505761373000107550010001200771315409772</t>
-  </si>
-  <si>
-    <t xml:space="preserve">64.914</t>
   </si>
   <si>
     <t xml:space="preserve">04/06/2026</t>
@@ -472,19 +454,10 @@
     <t xml:space="preserve">35260597837181002190550010050804131517661247</t>
   </si>
   <si>
-    <t xml:space="preserve">162.731</t>
+    <t xml:space="preserve">5.082.995</t>
   </si>
   <si>
     <t xml:space="preserve">13/05/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">48,67</t>
-  </si>
-  <si>
-    <t xml:space="preserve">42260597837181005378550010001627311454274477</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.082.995</t>
   </si>
   <si>
     <t xml:space="preserve">461,96</t>
@@ -511,21 +484,6 @@
     <t xml:space="preserve">42260575339051000141550080006388181323119663</t>
   </si>
   <si>
-    <t xml:space="preserve">10.718 - STELLA IMPORTACAO E EXPORTACAO DE LUMINARIAS LTDA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">292.997</t>
-  </si>
-  <si>
-    <t xml:space="preserve">497,70</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">42260510691158000370550010002929971371918584</t>
-  </si>
-  <si>
     <t xml:space="preserve">638.522</t>
   </si>
   <si>
@@ -536,6 +494,18 @@
   </si>
   <si>
     <t xml:space="preserve">42260575339051000141550080006385221064002290</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.705 - DOKA - INDUSTRIA E COMERCIO LTDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">62.258</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42260501136190000131550010000622581125328628</t>
   </si>
   <si>
     <t xml:space="preserve">639.834</t>
@@ -560,6 +530,24 @@
   </si>
   <si>
     <t xml:space="preserve">42260575339051000141550080006403161190056807</t>
+  </si>
+  <si>
+    <t xml:space="preserve">642.479</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/05/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18/05/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13/06/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.812,04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42260575339051000141550080006424791298308020</t>
   </si>
   <si>
     <t xml:space="preserve">Total geral</t>
@@ -16805,7 +16793,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:BM47"/>
+  <dimension ref="A1:BM46"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="0" width="18"/>
@@ -17368,7 +17356,7 @@
     </row>
     <row r="6" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="n">
-        <v>306535</v>
+        <v>306724</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>81</v>
@@ -17386,7 +17374,7 @@
         <v>83</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="J6" s="9" t="s">
         <v>78</v>
@@ -17395,31 +17383,31 @@
         <v>70</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>5384.2</v>
+        <v>976.79</v>
       </c>
       <c r="M6" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N6" s="12" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O6" s="12" t="n">
-        <v>5384.2</v>
+        <v>970.48</v>
       </c>
       <c r="P6" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q6" s="13" t="n">
-        <v>0.023054</v>
+        <v>0</v>
       </c>
       <c r="R6" s="12" t="n">
-        <v>28.62</v>
+        <v>0</v>
       </c>
       <c r="S6" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T6" s="14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="U6" s="15" t="s">
         <v>72</v>
@@ -17431,16 +17419,16 @@
         <v>73</v>
       </c>
       <c r="X6" s="9" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="Y6" s="12" t="n">
-        <v>0</v>
+        <v>6.31</v>
       </c>
       <c r="Z6" s="12" t="n">
-        <v>0</v>
+        <v>976.79</v>
       </c>
       <c r="AA6" s="12" t="n">
-        <v>0</v>
+        <v>68.38</v>
       </c>
       <c r="AB6" s="12" t="n">
         <v>0</v>
@@ -17509,7 +17497,7 @@
         <v>76</v>
       </c>
       <c r="AX6" s="10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AY6" s="14" t="s">
         <v>75</v>
@@ -17545,7 +17533,7 @@
         <v>78</v>
       </c>
       <c r="BJ6" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="BK6" s="9" t="s">
         <v>75</v>
@@ -17559,79 +17547,79 @@
     </row>
     <row r="7" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="n">
-        <v>306724</v>
+        <v>306823</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
       <c r="F7" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>66</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="K7" s="11" t="s">
         <v>70</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>976.79</v>
+        <v>5775.71</v>
       </c>
       <c r="M7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N7" s="12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O7" s="12" t="n">
-        <v>970.48</v>
+        <v>5510.71</v>
       </c>
       <c r="P7" s="12" t="n">
-        <v>0</v>
+        <v>265</v>
       </c>
       <c r="Q7" s="13" t="n">
         <v>0</v>
       </c>
       <c r="R7" s="12" t="n">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="S7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T7" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="U7" s="15" t="s">
         <v>72</v>
       </c>
       <c r="V7" s="12" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="W7" s="9" t="s">
         <v>73</v>
       </c>
       <c r="X7" s="9" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="Y7" s="12" t="n">
-        <v>6.31</v>
+        <v>0</v>
       </c>
       <c r="Z7" s="12" t="n">
-        <v>976.79</v>
+        <v>5775.71</v>
       </c>
       <c r="AA7" s="12" t="n">
-        <v>68.38</v>
+        <v>404.3</v>
       </c>
       <c r="AB7" s="12" t="n">
         <v>0</v>
@@ -17700,7 +17688,7 @@
         <v>76</v>
       </c>
       <c r="AX7" s="10" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="AY7" s="14" t="s">
         <v>75</v>
@@ -17750,7 +17738,7 @@
     </row>
     <row r="8" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="n">
-        <v>306823</v>
+        <v>306845</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>93</v>
@@ -17765,7 +17753,7 @@
         <v>66</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="I8" s="9" t="s">
         <v>69</v>
@@ -17777,7 +17765,7 @@
         <v>70</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>5775.71</v>
+        <v>935.55</v>
       </c>
       <c r="M8" s="12" t="n">
         <v>0</v>
@@ -17786,16 +17774,16 @@
         <v>1</v>
       </c>
       <c r="O8" s="12" t="n">
-        <v>5510.71</v>
+        <v>935.55</v>
       </c>
       <c r="P8" s="12" t="n">
-        <v>265</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="13" t="n">
         <v>0</v>
       </c>
       <c r="R8" s="12" t="n">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="S8" s="12" t="n">
         <v>0</v>
@@ -17807,7 +17795,7 @@
         <v>72</v>
       </c>
       <c r="V8" s="12" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="W8" s="9" t="s">
         <v>73</v>
@@ -17819,10 +17807,10 @@
         <v>0</v>
       </c>
       <c r="Z8" s="12" t="n">
-        <v>5775.71</v>
+        <v>935.55</v>
       </c>
       <c r="AA8" s="12" t="n">
-        <v>404.3</v>
+        <v>65.49</v>
       </c>
       <c r="AB8" s="12" t="n">
         <v>0</v>
@@ -17941,16 +17929,16 @@
     </row>
     <row r="9" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="n">
-        <v>306845</v>
+        <v>306869</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>66</v>
@@ -17959,16 +17947,16 @@
         <v>69</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>69</v>
+        <v>99</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="K9" s="11" t="s">
         <v>70</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>935.55</v>
+        <v>1725.01</v>
       </c>
       <c r="M9" s="12" t="n">
         <v>0</v>
@@ -17977,43 +17965,43 @@
         <v>1</v>
       </c>
       <c r="O9" s="12" t="n">
-        <v>935.55</v>
+        <v>1725.01</v>
       </c>
       <c r="P9" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q9" s="13" t="n">
-        <v>0</v>
+        <v>0.008288</v>
       </c>
       <c r="R9" s="12" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="S9" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T9" s="14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U9" s="15" t="s">
         <v>72</v>
       </c>
       <c r="V9" s="12" t="n">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="W9" s="9" t="s">
         <v>73</v>
       </c>
       <c r="X9" s="9" t="s">
-        <v>69</v>
+        <v>99</v>
       </c>
       <c r="Y9" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Z9" s="12" t="n">
-        <v>935.55</v>
+        <v>1725.01</v>
       </c>
       <c r="AA9" s="12" t="n">
-        <v>65.49</v>
+        <v>120.75</v>
       </c>
       <c r="AB9" s="12" t="n">
         <v>0</v>
@@ -18118,7 +18106,7 @@
         <v>78</v>
       </c>
       <c r="BJ9" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="BK9" s="9" t="s">
         <v>75</v>
@@ -18135,13 +18123,13 @@
         <v>306871</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
       <c r="F10" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>66</v>
@@ -18150,10 +18138,10 @@
         <v>69</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="K10" s="11" t="s">
         <v>70</v>
@@ -18183,7 +18171,7 @@
         <v>0</v>
       </c>
       <c r="T10" s="14" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="U10" s="15" t="s">
         <v>72</v>
@@ -18195,7 +18183,7 @@
         <v>73</v>
       </c>
       <c r="X10" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="Y10" s="12" t="n">
         <v>0</v>
@@ -18309,7 +18297,7 @@
         <v>78</v>
       </c>
       <c r="BJ10" s="9" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="BK10" s="9" t="s">
         <v>75</v>
@@ -18326,13 +18314,13 @@
         <v>306872</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
       <c r="F11" s="9" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>66</v>
@@ -18341,7 +18329,7 @@
         <v>69</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="J11" s="9" t="s">
         <v>78</v>
@@ -18374,7 +18362,7 @@
         <v>0</v>
       </c>
       <c r="T11" s="14" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="U11" s="15" t="s">
         <v>72</v>
@@ -18386,7 +18374,7 @@
         <v>73</v>
       </c>
       <c r="X11" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="Y11" s="12" t="n">
         <v>0</v>
@@ -18464,7 +18452,7 @@
         <v>76</v>
       </c>
       <c r="AX11" s="10" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="AY11" s="14" t="s">
         <v>75</v>
@@ -18500,7 +18488,7 @@
         <v>78</v>
       </c>
       <c r="BJ11" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="BK11" s="9" t="s">
         <v>75</v>
@@ -18517,13 +18505,13 @@
         <v>306873</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
       <c r="F12" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>66</v>
@@ -18532,10 +18520,10 @@
         <v>69</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="K12" s="11" t="s">
         <v>70</v>
@@ -18565,7 +18553,7 @@
         <v>0</v>
       </c>
       <c r="T12" s="14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="U12" s="15" t="s">
         <v>72</v>
@@ -18577,7 +18565,7 @@
         <v>73</v>
       </c>
       <c r="X12" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="Y12" s="12" t="n">
         <v>0</v>
@@ -18691,7 +18679,7 @@
         <v>78</v>
       </c>
       <c r="BJ12" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="BK12" s="9" t="s">
         <v>75</v>
@@ -18708,13 +18696,13 @@
         <v>306874</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
       <c r="F13" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G13" s="10" t="s">
         <v>66</v>
@@ -18723,10 +18711,10 @@
         <v>69</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="K13" s="11" t="s">
         <v>70</v>
@@ -18756,7 +18744,7 @@
         <v>0</v>
       </c>
       <c r="T13" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="U13" s="15" t="s">
         <v>72</v>
@@ -18768,7 +18756,7 @@
         <v>73</v>
       </c>
       <c r="X13" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="Y13" s="12" t="n">
         <v>0</v>
@@ -18882,7 +18870,7 @@
         <v>78</v>
       </c>
       <c r="BJ13" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="BK13" s="9" t="s">
         <v>75</v>
@@ -18899,13 +18887,13 @@
         <v>306875</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
       <c r="F14" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G14" s="10" t="s">
         <v>66</v>
@@ -18914,10 +18902,10 @@
         <v>69</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="K14" s="11" t="s">
         <v>70</v>
@@ -18947,7 +18935,7 @@
         <v>0</v>
       </c>
       <c r="T14" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="U14" s="15" t="s">
         <v>72</v>
@@ -18959,7 +18947,7 @@
         <v>73</v>
       </c>
       <c r="X14" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="Y14" s="12" t="n">
         <v>0</v>
@@ -19073,7 +19061,7 @@
         <v>78</v>
       </c>
       <c r="BJ14" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="BK14" s="9" t="s">
         <v>75</v>
@@ -19090,13 +19078,13 @@
         <v>306876</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
       <c r="F15" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G15" s="10" t="s">
         <v>66</v>
@@ -19105,10 +19093,10 @@
         <v>69</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="K15" s="11" t="s">
         <v>70</v>
@@ -19138,7 +19126,7 @@
         <v>0</v>
       </c>
       <c r="T15" s="14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="U15" s="15" t="s">
         <v>72</v>
@@ -19150,7 +19138,7 @@
         <v>73</v>
       </c>
       <c r="X15" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="Y15" s="12" t="n">
         <v>0</v>
@@ -19264,7 +19252,7 @@
         <v>78</v>
       </c>
       <c r="BJ15" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="BK15" s="9" t="s">
         <v>75</v>
@@ -19281,22 +19269,22 @@
         <v>306880</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
       <c r="F16" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="G16" s="10" t="s">
         <v>123</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>124</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>69</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="J16" s="9" t="s">
         <v>78</v>
@@ -19329,7 +19317,7 @@
         <v>0</v>
       </c>
       <c r="T16" s="14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="U16" s="15" t="s">
         <v>72</v>
@@ -19341,7 +19329,7 @@
         <v>73</v>
       </c>
       <c r="X16" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="Y16" s="12" t="n">
         <v>3.51</v>
@@ -19419,7 +19407,7 @@
         <v>76</v>
       </c>
       <c r="AX16" s="10" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="AY16" s="14" t="s">
         <v>75</v>
@@ -19455,7 +19443,7 @@
         <v>78</v>
       </c>
       <c r="BJ16" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="BK16" s="9" t="s">
         <v>75</v>
@@ -19469,79 +19457,79 @@
     </row>
     <row r="17" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="n">
-        <v>306969</v>
+        <v>306975</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>127</v>
+        <v>93</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
       <c r="F17" s="9" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G17" s="10" t="s">
         <v>66</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>69</v>
+        <v>99</v>
       </c>
       <c r="I17" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K17" s="11" t="s">
         <v>70</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>3625.8</v>
+        <v>985.72</v>
       </c>
       <c r="M17" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N17" s="12" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O17" s="12" t="n">
-        <v>3315.52</v>
+        <v>985.72</v>
       </c>
       <c r="P17" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q17" s="13" t="n">
-        <v>0</v>
+        <v>0.002368</v>
       </c>
       <c r="R17" s="12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S17" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T17" s="14" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="U17" s="15" t="s">
         <v>72</v>
       </c>
       <c r="V17" s="12" t="n">
-        <v>60.33</v>
+        <v>41.98</v>
       </c>
       <c r="W17" s="9" t="s">
         <v>73</v>
       </c>
       <c r="X17" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="Y17" s="12" t="n">
-        <v>310.28</v>
+        <v>0</v>
       </c>
       <c r="Z17" s="12" t="n">
-        <v>3315.52</v>
+        <v>985.72</v>
       </c>
       <c r="AA17" s="12" t="n">
-        <v>132.63</v>
+        <v>69</v>
       </c>
       <c r="AB17" s="12" t="n">
         <v>0</v>
@@ -19646,7 +19634,7 @@
         <v>78</v>
       </c>
       <c r="BJ17" s="9" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="BK17" s="9" t="s">
         <v>75</v>
@@ -19660,34 +19648,34 @@
     </row>
     <row r="18" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="n">
-        <v>306975</v>
+        <v>306976</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
       <c r="F18" s="9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="G18" s="10" t="s">
         <v>66</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="K18" s="11" t="s">
         <v>70</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>985.72</v>
+        <v>1478.58</v>
       </c>
       <c r="M18" s="12" t="n">
         <v>0</v>
@@ -19696,43 +19684,43 @@
         <v>1</v>
       </c>
       <c r="O18" s="12" t="n">
-        <v>985.72</v>
+        <v>1478.58</v>
       </c>
       <c r="P18" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q18" s="13" t="n">
-        <v>0.002368</v>
+        <v>0.007104</v>
       </c>
       <c r="R18" s="12" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="S18" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T18" s="14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="U18" s="15" t="s">
         <v>72</v>
       </c>
       <c r="V18" s="12" t="n">
-        <v>41.98</v>
+        <v>41.99</v>
       </c>
       <c r="W18" s="9" t="s">
         <v>73</v>
       </c>
       <c r="X18" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="Y18" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Z18" s="12" t="n">
-        <v>985.72</v>
+        <v>1478.58</v>
       </c>
       <c r="AA18" s="12" t="n">
-        <v>69</v>
+        <v>103.5</v>
       </c>
       <c r="AB18" s="12" t="n">
         <v>0</v>
@@ -19837,7 +19825,7 @@
         <v>78</v>
       </c>
       <c r="BJ18" s="9" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="BK18" s="9" t="s">
         <v>75</v>
@@ -19851,28 +19839,28 @@
     </row>
     <row r="19" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="n">
-        <v>306976</v>
+        <v>306977</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
       <c r="F19" s="9" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="G19" s="10" t="s">
         <v>66</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="K19" s="11" t="s">
         <v>70</v>
@@ -19902,7 +19890,7 @@
         <v>0</v>
       </c>
       <c r="T19" s="14" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="U19" s="15" t="s">
         <v>72</v>
@@ -19914,7 +19902,7 @@
         <v>73</v>
       </c>
       <c r="X19" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="Y19" s="12" t="n">
         <v>0</v>
@@ -20028,7 +20016,7 @@
         <v>78</v>
       </c>
       <c r="BJ19" s="9" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="BK19" s="9" t="s">
         <v>75</v>
@@ -20042,28 +20030,28 @@
     </row>
     <row r="20" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="n">
-        <v>306977</v>
+        <v>307040</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
       <c r="F20" s="9" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="G20" s="10" t="s">
         <v>66</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="K20" s="11" t="s">
         <v>70</v>
@@ -20093,7 +20081,7 @@
         <v>0</v>
       </c>
       <c r="T20" s="14" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="U20" s="15" t="s">
         <v>72</v>
@@ -20105,7 +20093,7 @@
         <v>73</v>
       </c>
       <c r="X20" s="9" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="Y20" s="12" t="n">
         <v>0</v>
@@ -20219,7 +20207,7 @@
         <v>78</v>
       </c>
       <c r="BJ20" s="9" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="BK20" s="9" t="s">
         <v>75</v>
@@ -20233,34 +20221,34 @@
     </row>
     <row r="21" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="n">
-        <v>307040</v>
+        <v>307172</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>98</v>
+        <v>139</v>
       </c>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
       <c r="F21" s="9" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G21" s="10" t="s">
         <v>66</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>134</v>
+        <v>78</v>
       </c>
       <c r="K21" s="11" t="s">
         <v>70</v>
       </c>
       <c r="L21" s="12" t="n">
-        <v>1478.58</v>
+        <v>404.81</v>
       </c>
       <c r="M21" s="12" t="n">
         <v>0</v>
@@ -20269,43 +20257,43 @@
         <v>1</v>
       </c>
       <c r="O21" s="12" t="n">
-        <v>1478.58</v>
+        <v>404.81</v>
       </c>
       <c r="P21" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q21" s="13" t="n">
-        <v>0.007104</v>
+        <v>0.000858</v>
       </c>
       <c r="R21" s="12" t="n">
-        <v>6</v>
+        <v>2.43</v>
       </c>
       <c r="S21" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T21" s="14" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="U21" s="15" t="s">
         <v>72</v>
       </c>
       <c r="V21" s="12" t="n">
-        <v>41.99</v>
+        <v>0</v>
       </c>
       <c r="W21" s="9" t="s">
         <v>73</v>
       </c>
       <c r="X21" s="9" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="Y21" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Z21" s="12" t="n">
-        <v>1478.58</v>
+        <v>404.81</v>
       </c>
       <c r="AA21" s="12" t="n">
-        <v>103.5</v>
+        <v>16.19</v>
       </c>
       <c r="AB21" s="12" t="n">
         <v>0</v>
@@ -20374,7 +20362,7 @@
         <v>76</v>
       </c>
       <c r="AX21" s="10" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="AY21" s="14" t="s">
         <v>75</v>
@@ -20410,7 +20398,7 @@
         <v>78</v>
       </c>
       <c r="BJ21" s="9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="BK21" s="9" t="s">
         <v>75</v>
@@ -20424,25 +20412,25 @@
     </row>
     <row r="22" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="n">
-        <v>307172</v>
+        <v>307219</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
       <c r="F22" s="9" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G22" s="10" t="s">
         <v>66</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="J22" s="9" t="s">
         <v>78</v>
@@ -20451,7 +20439,7 @@
         <v>70</v>
       </c>
       <c r="L22" s="12" t="n">
-        <v>404.81</v>
+        <v>461.96</v>
       </c>
       <c r="M22" s="12" t="n">
         <v>0</v>
@@ -20460,13 +20448,13 @@
         <v>1</v>
       </c>
       <c r="O22" s="12" t="n">
-        <v>404.81</v>
+        <v>461.96</v>
       </c>
       <c r="P22" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q22" s="13" t="n">
-        <v>0.000858</v>
+        <v>0.002057</v>
       </c>
       <c r="R22" s="12" t="n">
         <v>2.43</v>
@@ -20475,7 +20463,7 @@
         <v>0</v>
       </c>
       <c r="T22" s="14" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="U22" s="15" t="s">
         <v>72</v>
@@ -20487,16 +20475,16 @@
         <v>73</v>
       </c>
       <c r="X22" s="9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="Y22" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Z22" s="12" t="n">
-        <v>404.81</v>
+        <v>461.96</v>
       </c>
       <c r="AA22" s="12" t="n">
-        <v>16.19</v>
+        <v>18.48</v>
       </c>
       <c r="AB22" s="12" t="n">
         <v>0</v>
@@ -20565,7 +20553,7 @@
         <v>76</v>
       </c>
       <c r="AX22" s="10" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="AY22" s="14" t="s">
         <v>75</v>
@@ -20601,7 +20589,7 @@
         <v>78</v>
       </c>
       <c r="BJ22" s="9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="BK22" s="9" t="s">
         <v>75</v>
@@ -20615,34 +20603,34 @@
     </row>
     <row r="23" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="n">
-        <v>307205</v>
+        <v>307243</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>87</v>
+        <v>148</v>
       </c>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
       <c r="F23" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="G23" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="G23" s="10" t="s">
-        <v>66</v>
-      </c>
       <c r="H23" s="9" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="I23" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="J23" s="9" t="s">
         <v>151</v>
-      </c>
-      <c r="J23" s="9" t="s">
-        <v>78</v>
       </c>
       <c r="K23" s="11" t="s">
         <v>70</v>
       </c>
       <c r="L23" s="12" t="n">
-        <v>48.67</v>
+        <v>2077.92</v>
       </c>
       <c r="M23" s="12" t="n">
         <v>0</v>
@@ -20651,16 +20639,16 @@
         <v>1</v>
       </c>
       <c r="O23" s="12" t="n">
-        <v>48.36</v>
+        <v>2077.92</v>
       </c>
       <c r="P23" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q23" s="13" t="n">
-        <v>0.01185</v>
+        <v>0.007844</v>
       </c>
       <c r="R23" s="12" t="n">
-        <v>34.5</v>
+        <v>0.81</v>
       </c>
       <c r="S23" s="12" t="n">
         <v>0</v>
@@ -20672,22 +20660,22 @@
         <v>72</v>
       </c>
       <c r="V23" s="12" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="W23" s="9" t="s">
         <v>73</v>
       </c>
       <c r="X23" s="9" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="Y23" s="12" t="n">
-        <v>0.31</v>
+        <v>0</v>
       </c>
       <c r="Z23" s="12" t="n">
-        <v>48.36</v>
+        <v>2077.92</v>
       </c>
       <c r="AA23" s="12" t="n">
-        <v>3.39</v>
+        <v>145.45</v>
       </c>
       <c r="AB23" s="12" t="n">
         <v>0</v>
@@ -20756,7 +20744,7 @@
         <v>76</v>
       </c>
       <c r="AX23" s="10" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="AY23" s="14" t="s">
         <v>75</v>
@@ -20806,10 +20794,10 @@
     </row>
     <row r="24" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="n">
-        <v>307219</v>
+        <v>307294</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
@@ -20818,22 +20806,22 @@
         <v>154</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>66</v>
+        <v>150</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="I24" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="J24" s="9" t="s">
         <v>151</v>
-      </c>
-      <c r="J24" s="9" t="s">
-        <v>78</v>
       </c>
       <c r="K24" s="11" t="s">
         <v>70</v>
       </c>
       <c r="L24" s="12" t="n">
-        <v>461.96</v>
+        <v>4402.37</v>
       </c>
       <c r="M24" s="12" t="n">
         <v>0</v>
@@ -20842,43 +20830,43 @@
         <v>1</v>
       </c>
       <c r="O24" s="12" t="n">
-        <v>461.96</v>
+        <v>4402.37</v>
       </c>
       <c r="P24" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q24" s="13" t="n">
-        <v>0.002057</v>
+        <v>0</v>
       </c>
       <c r="R24" s="12" t="n">
-        <v>2.43</v>
+        <v>8.3</v>
       </c>
       <c r="S24" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T24" s="14" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="U24" s="15" t="s">
         <v>72</v>
       </c>
       <c r="V24" s="12" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="W24" s="9" t="s">
         <v>73</v>
       </c>
       <c r="X24" s="9" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="Y24" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Z24" s="12" t="n">
-        <v>461.96</v>
+        <v>4402.37</v>
       </c>
       <c r="AA24" s="12" t="n">
-        <v>18.48</v>
+        <v>308.17</v>
       </c>
       <c r="AB24" s="12" t="n">
         <v>0</v>
@@ -20947,7 +20935,7 @@
         <v>76</v>
       </c>
       <c r="AX24" s="10" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="AY24" s="14" t="s">
         <v>75</v>
@@ -20983,7 +20971,7 @@
         <v>78</v>
       </c>
       <c r="BJ24" s="9" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BK24" s="9" t="s">
         <v>75</v>
@@ -20997,34 +20985,34 @@
     </row>
     <row r="25" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="n">
-        <v>307243</v>
+        <v>307310</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>159</v>
+        <v>66</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>160</v>
+        <v>78</v>
       </c>
       <c r="K25" s="11" t="s">
         <v>70</v>
       </c>
       <c r="L25" s="12" t="n">
-        <v>2077.92</v>
+        <v>30</v>
       </c>
       <c r="M25" s="12" t="n">
         <v>0</v>
@@ -21033,43 +21021,43 @@
         <v>1</v>
       </c>
       <c r="O25" s="12" t="n">
-        <v>2077.92</v>
+        <v>30</v>
       </c>
       <c r="P25" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q25" s="13" t="n">
-        <v>0.007844</v>
+        <v>0</v>
       </c>
       <c r="R25" s="12" t="n">
-        <v>0.81</v>
+        <v>38</v>
       </c>
       <c r="S25" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T25" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="U25" s="15" t="s">
         <v>72</v>
       </c>
       <c r="V25" s="12" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="W25" s="9" t="s">
         <v>73</v>
       </c>
       <c r="X25" s="9" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="Y25" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Z25" s="12" t="n">
-        <v>2077.92</v>
+        <v>30</v>
       </c>
       <c r="AA25" s="12" t="n">
-        <v>145.45</v>
+        <v>1.2</v>
       </c>
       <c r="AB25" s="12" t="n">
         <v>0</v>
@@ -21138,7 +21126,7 @@
         <v>76</v>
       </c>
       <c r="AX25" s="10" t="s">
-        <v>77</v>
+        <v>107</v>
       </c>
       <c r="AY25" s="14" t="s">
         <v>75</v>
@@ -21174,7 +21162,7 @@
         <v>78</v>
       </c>
       <c r="BJ25" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="BK25" s="9" t="s">
         <v>75</v>
@@ -21188,34 +21176,34 @@
     </row>
     <row r="26" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="n">
-        <v>307275</v>
+        <v>307332</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="C26" s="9"/>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
       <c r="F26" s="9" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>66</v>
+        <v>150</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>78</v>
+        <v>163</v>
       </c>
       <c r="K26" s="11" t="s">
         <v>70</v>
       </c>
       <c r="L26" s="12" t="n">
-        <v>497.7</v>
+        <v>1494.11</v>
       </c>
       <c r="M26" s="12" t="n">
         <v>0</v>
@@ -21224,43 +21212,43 @@
         <v>1</v>
       </c>
       <c r="O26" s="12" t="n">
-        <v>497.7</v>
+        <v>1494.11</v>
       </c>
       <c r="P26" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q26" s="13" t="n">
-        <v>0</v>
+        <v>0.002473</v>
       </c>
       <c r="R26" s="12" t="n">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="S26" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T26" s="14" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="U26" s="15" t="s">
         <v>72</v>
       </c>
       <c r="V26" s="12" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="W26" s="9" t="s">
         <v>73</v>
       </c>
       <c r="X26" s="9" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="Y26" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Z26" s="12" t="n">
-        <v>497.7</v>
+        <v>1494.11</v>
       </c>
       <c r="AA26" s="12" t="n">
-        <v>19.91</v>
+        <v>104.59</v>
       </c>
       <c r="AB26" s="12" t="n">
         <v>0</v>
@@ -21326,10 +21314,10 @@
         <v>74</v>
       </c>
       <c r="AW26" s="14" t="s">
-        <v>166</v>
+        <v>76</v>
       </c>
       <c r="AX26" s="10" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="AY26" s="14" t="s">
         <v>75</v>
@@ -21365,7 +21353,7 @@
         <v>78</v>
       </c>
       <c r="BJ26" s="9" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="BK26" s="9" t="s">
         <v>75</v>
@@ -21379,34 +21367,34 @@
     </row>
     <row r="27" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="n">
-        <v>307294</v>
+        <v>307348</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="C27" s="9"/>
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
       <c r="F27" s="9" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="K27" s="11" t="s">
         <v>70</v>
       </c>
       <c r="L27" s="12" t="n">
-        <v>4402.37</v>
+        <v>1360.01</v>
       </c>
       <c r="M27" s="12" t="n">
         <v>0</v>
@@ -21415,22 +21403,22 @@
         <v>1</v>
       </c>
       <c r="O27" s="12" t="n">
-        <v>4402.37</v>
+        <v>1277</v>
       </c>
       <c r="P27" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q27" s="13" t="n">
-        <v>0</v>
+        <v>0.013954</v>
       </c>
       <c r="R27" s="12" t="n">
-        <v>8.3</v>
+        <v>1.78</v>
       </c>
       <c r="S27" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T27" s="14" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="U27" s="15" t="s">
         <v>72</v>
@@ -21442,16 +21430,16 @@
         <v>73</v>
       </c>
       <c r="X27" s="9" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
       <c r="Y27" s="12" t="n">
-        <v>0</v>
+        <v>83.01</v>
       </c>
       <c r="Z27" s="12" t="n">
-        <v>4402.37</v>
+        <v>1277</v>
       </c>
       <c r="AA27" s="12" t="n">
-        <v>308.17</v>
+        <v>89.39</v>
       </c>
       <c r="AB27" s="12" t="n">
         <v>0</v>
@@ -21556,7 +21544,7 @@
         <v>78</v>
       </c>
       <c r="BJ27" s="9" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="BK27" s="9" t="s">
         <v>75</v>
@@ -21570,25 +21558,25 @@
     </row>
     <row r="28" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="n">
-        <v>307332</v>
+        <v>307432</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="C28" s="9"/>
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
       <c r="F28" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="G28" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="I28" s="9" t="s">
         <v>172</v>
-      </c>
-      <c r="G28" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="H28" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="I28" s="9" t="s">
-        <v>169</v>
       </c>
       <c r="J28" s="9" t="s">
         <v>173</v>
@@ -21597,7 +21585,7 @@
         <v>70</v>
       </c>
       <c r="L28" s="12" t="n">
-        <v>1494.11</v>
+        <v>2812.04</v>
       </c>
       <c r="M28" s="12" t="n">
         <v>0</v>
@@ -21606,16 +21594,16 @@
         <v>1</v>
       </c>
       <c r="O28" s="12" t="n">
-        <v>1494.11</v>
+        <v>2812.04</v>
       </c>
       <c r="P28" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q28" s="13" t="n">
-        <v>0.002473</v>
+        <v>0.007844</v>
       </c>
       <c r="R28" s="12" t="n">
-        <v>0.77</v>
+        <v>1.78</v>
       </c>
       <c r="S28" s="12" t="n">
         <v>0</v>
@@ -21633,16 +21621,16 @@
         <v>73</v>
       </c>
       <c r="X28" s="9" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="Y28" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Z28" s="12" t="n">
-        <v>1494.11</v>
+        <v>2812.04</v>
       </c>
       <c r="AA28" s="12" t="n">
-        <v>104.59</v>
+        <v>196.84</v>
       </c>
       <c r="AB28" s="12" t="n">
         <v>0</v>
@@ -21760,518 +21748,396 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8" t="n">
-        <v>307348</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9" t="s">
+      <c r="A29" s="4"/>
+    </row>
+    <row r="30" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="17" t="s">
         <v>176</v>
       </c>
-      <c r="G29" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="H29" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="I29" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="J29" s="9" t="s">
-        <v>177</v>
-      </c>
-      <c r="K29" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="L29" s="12" t="n">
-        <v>1360.01</v>
-      </c>
-      <c r="M29" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="O29" s="12" t="n">
-        <v>1277</v>
-      </c>
-      <c r="P29" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q29" s="13" t="n">
-        <v>0.013954</v>
-      </c>
-      <c r="R29" s="12" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="S29" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T29" s="14" t="s">
-        <v>178</v>
-      </c>
-      <c r="U29" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="V29" s="12" t="n">
-        <v>28</v>
-      </c>
-      <c r="W29" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="X29" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="Y29" s="12" t="n">
-        <v>83.01</v>
-      </c>
-      <c r="Z29" s="12" t="n">
-        <v>1277</v>
-      </c>
-      <c r="AA29" s="12" t="n">
-        <v>89.39</v>
-      </c>
-      <c r="AB29" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC29" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD29" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE29" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF29" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG29" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH29" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="AI29" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ29" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK29" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL29" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM29" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="AN29" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="AO29" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="AP29" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="AQ29" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="AR29" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="AS29" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="AT29" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="AU29" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="AV29" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="AW29" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="AX29" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="AY29" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="AZ29" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="BA29" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="BB29" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="BC29" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="BD29" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="BE29" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="BF29" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="BG29" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="BH29" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="BI29" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="BJ29" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="BK29" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="BL29" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="BM29" s="16" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="17"/>
+      <c r="H30" s="17"/>
+      <c r="I30" s="17"/>
+      <c r="J30" s="17"/>
+      <c r="K30" s="17"/>
+      <c r="L30" s="17"/>
+      <c r="M30" s="17"/>
+      <c r="N30" s="17"/>
+      <c r="O30" s="17"/>
+      <c r="P30" s="17"/>
+      <c r="Q30" s="17"/>
+      <c r="R30" s="17"/>
+      <c r="S30" s="17"/>
+      <c r="T30" s="17"/>
+      <c r="U30" s="17"/>
+      <c r="V30" s="17"/>
     </row>
     <row r="31" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="18" t="s">
+        <v>177</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="D31" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="E31" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="F31" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="G31" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="H31" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="I31" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="J31" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="K31" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="L31" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="M31" s="18" t="s">
         <v>180</v>
       </c>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="17"/>
-      <c r="I31" s="17"/>
-      <c r="J31" s="17"/>
-      <c r="K31" s="17"/>
-      <c r="L31" s="17"/>
-      <c r="M31" s="17"/>
-      <c r="N31" s="17"/>
-      <c r="O31" s="17"/>
-      <c r="P31" s="17"/>
-      <c r="Q31" s="17"/>
-      <c r="R31" s="17"/>
-      <c r="S31" s="17"/>
-      <c r="T31" s="17"/>
-      <c r="U31" s="17"/>
-      <c r="V31" s="17"/>
+      <c r="N31" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="O31" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="P31" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q31" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="R31" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="S31" s="18" t="s">
+        <v>181</v>
+      </c>
+      <c r="T31" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="U31" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="V31" s="18" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="32" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="18" t="s">
-        <v>181</v>
-      </c>
-      <c r="B32" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="C32" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="D32" s="18" t="s">
-        <v>182</v>
-      </c>
-      <c r="E32" s="18" t="s">
+    <row r="32" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="19" t="n">
         <v>24</v>
       </c>
-      <c r="F32" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="G32" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="H32" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="I32" s="18" t="s">
+      <c r="B32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="19" t="n">
+        <v>265</v>
+      </c>
+      <c r="D32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="19" t="n">
+        <v>92.83</v>
+      </c>
+      <c r="F32" s="19" t="n">
+        <v>50365.02</v>
+      </c>
+      <c r="G32" s="19" t="n">
+        <v>3394.43</v>
+      </c>
+      <c r="H32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="19" t="n">
+        <v>50451.54</v>
+      </c>
+      <c r="L32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" s="20" t="n">
+        <v>0.141296</v>
+      </c>
+      <c r="S32" s="19" t="n">
+        <v>50093.71</v>
+      </c>
+      <c r="T32" s="19" t="n">
+        <v>50451.54</v>
+      </c>
+      <c r="U32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="V32" s="19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C33" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="D33" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="E33" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="F33" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="G33" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="H33" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="I33" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="J33" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="K33" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="J32" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="K32" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="L32" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="M32" s="18" t="s">
+      <c r="L33" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="N32" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="O32" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="P32" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q32" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="R32" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="S32" s="18" t="s">
+      <c r="M33" s="18" t="s">
         <v>185</v>
       </c>
-      <c r="T32" s="18" t="s">
-        <v>186</v>
-      </c>
-      <c r="U32" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="V32" s="18" t="s">
-        <v>37</v>
-      </c>
     </row>
-    <row r="33" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="19" t="n">
-        <v>25</v>
-      </c>
-      <c r="B33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C33" s="19" t="n">
-        <v>265</v>
-      </c>
-      <c r="D33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="19" t="n">
-        <v>403.42</v>
-      </c>
-      <c r="F33" s="19" t="n">
-        <v>49659.55</v>
-      </c>
-      <c r="G33" s="19" t="n">
-        <v>3231.57</v>
-      </c>
-      <c r="H33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" s="19" t="n">
-        <v>55440.86</v>
-      </c>
-      <c r="L33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="R33" s="20" t="n">
-        <v>0.160068</v>
-      </c>
-      <c r="S33" s="19" t="n">
-        <v>54772.44</v>
-      </c>
-      <c r="T33" s="19" t="n">
-        <v>55440.86</v>
-      </c>
-      <c r="U33" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="V33" s="19" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="B34" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="C34" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="D34" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="E34" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="F34" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="G34" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="H34" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="I34" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="J34" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="K34" s="18" t="s">
-        <v>187</v>
-      </c>
-      <c r="L34" s="18" t="s">
-        <v>188</v>
-      </c>
-      <c r="M34" s="18" t="s">
-        <v>189</v>
+    <row r="34" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="19" t="n">
+        <v>176.79</v>
+      </c>
+      <c r="B34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="19" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="E34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="19" t="n">
-        <v>193.12</v>
-      </c>
-      <c r="B35" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C35" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" s="19" t="n">
-        <v>31.81</v>
-      </c>
-      <c r="E35" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" s="19" t="n">
-        <v>0</v>
-      </c>
+      <c r="A35" s="4"/>
     </row>
-    <row r="36" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4"/>
+    <row r="36" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
+      <c r="G36" s="21"/>
+      <c r="H36" s="21"/>
+      <c r="I36" s="21"/>
+      <c r="J36" s="21"/>
+      <c r="K36" s="21"/>
+      <c r="L36" s="21"/>
+      <c r="M36" s="21"/>
+      <c r="N36" s="21"/>
+      <c r="O36" s="21"/>
+      <c r="P36" s="21"/>
+      <c r="Q36" s="21"/>
+      <c r="R36" s="21"/>
+      <c r="S36" s="21"/>
+      <c r="T36" s="21"/>
+      <c r="U36" s="21"/>
+      <c r="V36" s="21"/>
+      <c r="W36" s="21"/>
+      <c r="X36" s="21"/>
+      <c r="Y36" s="21"/>
+      <c r="Z36" s="21"/>
+      <c r="AA36" s="21"/>
+      <c r="AB36" s="21"/>
+      <c r="AC36" s="21"/>
+      <c r="AD36" s="21"/>
+      <c r="AE36" s="21"/>
+      <c r="AF36" s="21"/>
+      <c r="AG36" s="21"/>
+      <c r="AH36" s="21"/>
+      <c r="AI36" s="21"/>
+      <c r="AJ36" s="21"/>
+      <c r="AK36" s="21"/>
+      <c r="AL36" s="21"/>
+      <c r="AM36" s="21"/>
+      <c r="AN36" s="21"/>
+      <c r="AO36" s="21"/>
+      <c r="AP36" s="21"/>
+      <c r="AQ36" s="21"/>
+      <c r="AR36" s="21"/>
+      <c r="AS36" s="21"/>
+      <c r="AT36" s="21"/>
+      <c r="AU36" s="21"/>
+      <c r="AV36" s="21"/>
+      <c r="AW36" s="21"/>
+      <c r="AX36" s="21"/>
+      <c r="AY36" s="21"/>
+      <c r="AZ36" s="21"/>
+      <c r="BA36" s="21"/>
+      <c r="BB36" s="21"/>
+      <c r="BC36" s="21"/>
+      <c r="BD36" s="21"/>
+      <c r="BE36" s="21"/>
+      <c r="BF36" s="21"/>
+      <c r="BG36" s="21"/>
+      <c r="BH36" s="21"/>
+      <c r="BI36" s="21"/>
+      <c r="BJ36" s="21"/>
+      <c r="BK36" s="21"/>
+      <c r="BL36" s="21"/>
+      <c r="BM36" s="21"/>
     </row>
-    <row r="37" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="21" t="s">
-        <v>190</v>
-      </c>
-      <c r="B37" s="21"/>
-      <c r="C37" s="21"/>
-      <c r="D37" s="21"/>
-      <c r="E37" s="21"/>
-      <c r="F37" s="21"/>
-      <c r="G37" s="21"/>
-      <c r="H37" s="21"/>
-      <c r="I37" s="21"/>
-      <c r="J37" s="21"/>
-      <c r="K37" s="21"/>
-      <c r="L37" s="21"/>
-      <c r="M37" s="21"/>
-      <c r="N37" s="21"/>
-      <c r="O37" s="21"/>
-      <c r="P37" s="21"/>
-      <c r="Q37" s="21"/>
-      <c r="R37" s="21"/>
-      <c r="S37" s="21"/>
-      <c r="T37" s="21"/>
-      <c r="U37" s="21"/>
-      <c r="V37" s="21"/>
-      <c r="W37" s="21"/>
-      <c r="X37" s="21"/>
-      <c r="Y37" s="21"/>
-      <c r="Z37" s="21"/>
-      <c r="AA37" s="21"/>
-      <c r="AB37" s="21"/>
-      <c r="AC37" s="21"/>
-      <c r="AD37" s="21"/>
-      <c r="AE37" s="21"/>
-      <c r="AF37" s="21"/>
-      <c r="AG37" s="21"/>
-      <c r="AH37" s="21"/>
-      <c r="AI37" s="21"/>
-      <c r="AJ37" s="21"/>
-      <c r="AK37" s="21"/>
-      <c r="AL37" s="21"/>
-      <c r="AM37" s="21"/>
-      <c r="AN37" s="21"/>
-      <c r="AO37" s="21"/>
-      <c r="AP37" s="21"/>
-      <c r="AQ37" s="21"/>
-      <c r="AR37" s="21"/>
-      <c r="AS37" s="21"/>
-      <c r="AT37" s="21"/>
-      <c r="AU37" s="21"/>
-      <c r="AV37" s="21"/>
-      <c r="AW37" s="21"/>
-      <c r="AX37" s="21"/>
-      <c r="AY37" s="21"/>
-      <c r="AZ37" s="21"/>
-      <c r="BA37" s="21"/>
-      <c r="BB37" s="21"/>
-      <c r="BC37" s="21"/>
-      <c r="BD37" s="21"/>
-      <c r="BE37" s="21"/>
-      <c r="BF37" s="21"/>
-      <c r="BG37" s="21"/>
-      <c r="BH37" s="21"/>
-      <c r="BI37" s="21"/>
-      <c r="BJ37" s="21"/>
-      <c r="BK37" s="21"/>
-      <c r="BL37" s="21"/>
-      <c r="BM37" s="21"/>
+    <row r="37" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="4"/>
+      <c r="I37" s="4"/>
+      <c r="J37" s="4"/>
+      <c r="K37" s="4"/>
+      <c r="L37" s="4"/>
+      <c r="M37" s="4"/>
+      <c r="N37" s="4"/>
+      <c r="O37" s="4"/>
+      <c r="P37" s="4"/>
+      <c r="Q37" s="4"/>
+      <c r="R37" s="4"/>
+      <c r="S37" s="4"/>
+      <c r="T37" s="4"/>
+      <c r="U37" s="4"/>
+      <c r="V37" s="4"/>
+      <c r="W37" s="4"/>
+      <c r="X37" s="4"/>
+      <c r="Y37" s="4"/>
+      <c r="Z37" s="4"/>
+      <c r="AA37" s="4"/>
+      <c r="AB37" s="4"/>
+      <c r="AC37" s="4"/>
+      <c r="AD37" s="4"/>
+      <c r="AE37" s="4"/>
+      <c r="AF37" s="4"/>
+      <c r="AG37" s="4"/>
+      <c r="AH37" s="4"/>
+      <c r="AI37" s="4"/>
+      <c r="AJ37" s="4"/>
+      <c r="AK37" s="4"/>
+      <c r="AL37" s="4"/>
+      <c r="AM37" s="4"/>
+      <c r="AN37" s="4"/>
+      <c r="AO37" s="4"/>
+      <c r="AP37" s="4"/>
+      <c r="AQ37" s="4"/>
+      <c r="AR37" s="4"/>
+      <c r="AS37" s="4"/>
+      <c r="AT37" s="4"/>
+      <c r="AU37" s="4"/>
+      <c r="AV37" s="4"/>
+      <c r="AW37" s="4"/>
+      <c r="AX37" s="4"/>
+      <c r="AY37" s="4"/>
+      <c r="AZ37" s="4"/>
+      <c r="BA37" s="4"/>
+      <c r="BB37" s="4"/>
+      <c r="BC37" s="4"/>
+      <c r="BD37" s="4"/>
+      <c r="BE37" s="4"/>
+      <c r="BF37" s="4"/>
+      <c r="BG37" s="4"/>
+      <c r="BH37" s="4"/>
+      <c r="BI37" s="4"/>
+      <c r="BJ37" s="4"/>
+      <c r="BK37" s="4"/>
+      <c r="BL37" s="4"/>
+      <c r="BM37" s="4"/>
     </row>
     <row r="38" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>75</v>
+        <v>187</v>
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -22340,7 +22206,7 @@
     </row>
     <row r="39" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -22409,7 +22275,7 @@
     </row>
     <row r="40" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -22478,7 +22344,7 @@
     </row>
     <row r="41" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -22547,7 +22413,7 @@
     </row>
     <row r="42" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>22</v>
+        <v>190</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -22616,7 +22482,7 @@
     </row>
     <row r="43" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -22685,7 +22551,7 @@
     </row>
     <row r="44" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -22754,7 +22620,7 @@
     </row>
     <row r="45" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -22823,7 +22689,7 @@
     </row>
     <row r="46" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -22890,77 +22756,8 @@
       <c r="BL46" s="4"/>
       <c r="BM46" s="4"/>
     </row>
-    <row r="47" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="B47" s="4"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="4"/>
-      <c r="E47" s="4"/>
-      <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4"/>
-      <c r="I47" s="4"/>
-      <c r="J47" s="4"/>
-      <c r="K47" s="4"/>
-      <c r="L47" s="4"/>
-      <c r="M47" s="4"/>
-      <c r="N47" s="4"/>
-      <c r="O47" s="4"/>
-      <c r="P47" s="4"/>
-      <c r="Q47" s="4"/>
-      <c r="R47" s="4"/>
-      <c r="S47" s="4"/>
-      <c r="T47" s="4"/>
-      <c r="U47" s="4"/>
-      <c r="V47" s="4"/>
-      <c r="W47" s="4"/>
-      <c r="X47" s="4"/>
-      <c r="Y47" s="4"/>
-      <c r="Z47" s="4"/>
-      <c r="AA47" s="4"/>
-      <c r="AB47" s="4"/>
-      <c r="AC47" s="4"/>
-      <c r="AD47" s="4"/>
-      <c r="AE47" s="4"/>
-      <c r="AF47" s="4"/>
-      <c r="AG47" s="4"/>
-      <c r="AH47" s="4"/>
-      <c r="AI47" s="4"/>
-      <c r="AJ47" s="4"/>
-      <c r="AK47" s="4"/>
-      <c r="AL47" s="4"/>
-      <c r="AM47" s="4"/>
-      <c r="AN47" s="4"/>
-      <c r="AO47" s="4"/>
-      <c r="AP47" s="4"/>
-      <c r="AQ47" s="4"/>
-      <c r="AR47" s="4"/>
-      <c r="AS47" s="4"/>
-      <c r="AT47" s="4"/>
-      <c r="AU47" s="4"/>
-      <c r="AV47" s="4"/>
-      <c r="AW47" s="4"/>
-      <c r="AX47" s="4"/>
-      <c r="AY47" s="4"/>
-      <c r="AZ47" s="4"/>
-      <c r="BA47" s="4"/>
-      <c r="BB47" s="4"/>
-      <c r="BC47" s="4"/>
-      <c r="BD47" s="4"/>
-      <c r="BE47" s="4"/>
-      <c r="BF47" s="4"/>
-      <c r="BG47" s="4"/>
-      <c r="BH47" s="4"/>
-      <c r="BI47" s="4"/>
-      <c r="BJ47" s="4"/>
-      <c r="BK47" s="4"/>
-      <c r="BL47" s="4"/>
-      <c r="BM47" s="4"/>
-    </row>
   </sheetData>
-  <mergeCells count="41">
+  <mergeCells count="40">
     <mergeCell ref="A1:BI1"/>
     <mergeCell ref="BJ1:BM1"/>
     <mergeCell ref="A2:BM2"/>
@@ -22989,8 +22786,8 @@
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B28:E28"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="A31:V31"/>
+    <mergeCell ref="A30:V30"/>
+    <mergeCell ref="A36:BM36"/>
     <mergeCell ref="A37:BM37"/>
     <mergeCell ref="A38:BM38"/>
     <mergeCell ref="A39:BM39"/>
@@ -23001,7 +22798,6 @@
     <mergeCell ref="A44:BM44"/>
     <mergeCell ref="A45:BM45"/>
     <mergeCell ref="A46:BM46"/>
-    <mergeCell ref="A47:BM47"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
atualização banco + relatório supervisores
</commit_message>
<xml_diff>
--- a/tratando_tabelas/finitura/entradas_finitura.xlsx
+++ b/tratando_tabelas/finitura/entradas_finitura.xlsx
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="156">
   <si>
     <t xml:space="preserve">Santri ADM 1.1.5.8 R1</t>
   </si>
   <si>
-    <t xml:space="preserve">Emitido em: 22/06/2026 04:30:29</t>
+    <t xml:space="preserve">Emitido em: 23/06/2026 04:30:38</t>
   </si>
   <si>
     <t xml:space="preserve">Relação de entradas - Sintético</t>
@@ -226,16 +226,16 @@
     <t xml:space="preserve">Fornecedor substituto tributário</t>
   </si>
   <si>
-    <t xml:space="preserve">21.134 - NISSILIGHT COMERCIAL DE MATERIAIS ELETRICOS LTDA</t>
+    <t xml:space="preserve">761 - DOCOL FV IND.E COM. DE METAIS SANITARIOS LTDA</t>
   </si>
   <si>
-    <t xml:space="preserve">114.612</t>
+    <t xml:space="preserve">665.742</t>
   </si>
   <si>
-    <t xml:space="preserve">2</t>
+    <t xml:space="preserve">8</t>
   </si>
   <si>
-    <t xml:space="preserve">10/06/2026</t>
+    <t xml:space="preserve">12/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">16/06/2026</t>
@@ -247,7 +247,7 @@
     <t xml:space="preserve">XML</t>
   </si>
   <si>
-    <t xml:space="preserve">64.187,37</t>
+    <t xml:space="preserve">2.922,60</t>
   </si>
   <si>
     <t xml:space="preserve">Ag. chegada da mercadoria</t>
@@ -268,28 +268,10 @@
     <t xml:space="preserve">          </t>
   </si>
   <si>
-    <t xml:space="preserve">42260635635346000140550020001146121910680221</t>
+    <t xml:space="preserve">42260675339051000141550080006657421040310096</t>
   </si>
   <si>
     <t xml:space="preserve">Não</t>
-  </si>
-  <si>
-    <t xml:space="preserve">761 - DOCOL FV IND.E COM. DE METAIS SANITARIOS LTDA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">665.742</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12/06/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.922,60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">42260675339051000141550080006657421040310096</t>
   </si>
   <si>
     <t xml:space="preserve">22.015 - FOCO METALLO FABRICACAO E MONTAGEM DE LUMINARIAS E COMERCIO</t>
@@ -346,7 +328,13 @@
     <t xml:space="preserve">42260675339051000141550080006681221019457049</t>
   </si>
   <si>
+    <t xml:space="preserve">21.134 - NISSILIGHT COMERCIAL DE MATERIAIS ELETRICOS LTDA</t>
+  </si>
+  <si>
     <t xml:space="preserve">115.090</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
   </si>
   <si>
     <t xml:space="preserve">16/07/2026</t>
@@ -416,6 +404,24 @@
   </si>
   <si>
     <t xml:space="preserve">35260611389565000200570050004014491000878201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.705 - DOKA - INDUSTRIA E COMERCIO LTDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">63.920</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22/06/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20/07/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.432,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42260601136190000131550010000639201764544670</t>
   </si>
   <si>
     <t xml:space="preserve">Total geral</t>
@@ -17604,7 +17610,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="n">
-        <v>309190</v>
+        <v>309226</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>68</v>
@@ -17631,25 +17637,25 @@
         <v>74</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>64187.37</v>
+        <v>2922.6</v>
       </c>
       <c r="M5" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N5" s="12" t="n">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="O5" s="12" t="n">
-        <v>58730.21</v>
+        <v>2922.6</v>
       </c>
       <c r="P5" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q5" s="13" t="n">
-        <v>0</v>
+        <v>0.000744</v>
       </c>
       <c r="R5" s="12" t="n">
-        <v>2.5</v>
+        <v>2.18</v>
       </c>
       <c r="S5" s="12" t="n">
         <v>0</v>
@@ -17661,19 +17667,19 @@
         <v>76</v>
       </c>
       <c r="V5" s="12" t="n">
-        <v>51165.75</v>
+        <v>2466.6</v>
       </c>
       <c r="W5" s="12" t="n">
-        <v>51.17</v>
+        <v>2.47</v>
       </c>
       <c r="X5" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y5" s="12" t="n">
-        <v>460.49</v>
+        <v>22.2</v>
       </c>
       <c r="Z5" s="12" t="n">
-        <v>84.9</v>
+        <v>28</v>
       </c>
       <c r="AA5" s="9" t="s">
         <v>77</v>
@@ -17682,13 +17688,13 @@
         <v>72</v>
       </c>
       <c r="AC5" s="12" t="n">
-        <v>5457.16</v>
+        <v>0</v>
       </c>
       <c r="AD5" s="12" t="n">
-        <v>58730.21</v>
+        <v>2922.6</v>
       </c>
       <c r="AE5" s="12" t="n">
-        <v>2349.21</v>
+        <v>204.58</v>
       </c>
       <c r="AF5" s="12" t="n">
         <v>0</v>
@@ -17807,7 +17813,7 @@
     </row>
     <row r="6" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="n">
-        <v>309226</v>
+        <v>309242</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>84</v>
@@ -17828,13 +17834,13 @@
         <v>72</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="K6" s="11" t="s">
         <v>74</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>2922.6</v>
+        <v>1731.85</v>
       </c>
       <c r="M6" s="12" t="n">
         <v>0</v>
@@ -17843,40 +17849,40 @@
         <v>2</v>
       </c>
       <c r="O6" s="12" t="n">
-        <v>2922.6</v>
+        <v>1578</v>
       </c>
       <c r="P6" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q6" s="13" t="n">
-        <v>0.000744</v>
+        <v>0.5292</v>
       </c>
       <c r="R6" s="12" t="n">
-        <v>2.18</v>
+        <v>0</v>
       </c>
       <c r="S6" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T6" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="U6" s="15" t="s">
         <v>76</v>
       </c>
       <c r="V6" s="12" t="n">
-        <v>2466.6</v>
+        <v>1409.94</v>
       </c>
       <c r="W6" s="12" t="n">
-        <v>2.47</v>
+        <v>1.41</v>
       </c>
       <c r="X6" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y6" s="12" t="n">
-        <v>22.2</v>
+        <v>12.68</v>
       </c>
       <c r="Z6" s="12" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="AA6" s="9" t="s">
         <v>77</v>
@@ -17885,13 +17891,13 @@
         <v>72</v>
       </c>
       <c r="AC6" s="12" t="n">
-        <v>0</v>
+        <v>153.85</v>
       </c>
       <c r="AD6" s="12" t="n">
-        <v>2922.6</v>
+        <v>1578</v>
       </c>
       <c r="AE6" s="12" t="n">
-        <v>204.58</v>
+        <v>110.46</v>
       </c>
       <c r="AF6" s="12" t="n">
         <v>0</v>
@@ -17996,7 +18002,7 @@
         <v>81</v>
       </c>
       <c r="BN6" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="BO6" s="9" t="s">
         <v>79</v>
@@ -18010,19 +18016,19 @@
     </row>
     <row r="7" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="n">
-        <v>309242</v>
+        <v>309276</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
       <c r="F7" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>93</v>
@@ -18037,25 +18043,25 @@
         <v>74</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>1731.85</v>
+        <v>1299.12</v>
       </c>
       <c r="M7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N7" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O7" s="12" t="n">
-        <v>1578</v>
+        <v>1299.12</v>
       </c>
       <c r="P7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q7" s="13" t="n">
-        <v>0.5292</v>
+        <v>0</v>
       </c>
       <c r="R7" s="12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S7" s="12" t="n">
         <v>0</v>
@@ -18067,19 +18073,19 @@
         <v>76</v>
       </c>
       <c r="V7" s="12" t="n">
-        <v>1409.94</v>
+        <v>1367.5</v>
       </c>
       <c r="W7" s="12" t="n">
-        <v>1.41</v>
+        <v>1.37</v>
       </c>
       <c r="X7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y7" s="12" t="n">
-        <v>12.68</v>
+        <v>12.31</v>
       </c>
       <c r="Z7" s="12" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="AA7" s="9" t="s">
         <v>77</v>
@@ -18088,13 +18094,13 @@
         <v>72</v>
       </c>
       <c r="AC7" s="12" t="n">
-        <v>153.85</v>
+        <v>0</v>
       </c>
       <c r="AD7" s="12" t="n">
-        <v>1578</v>
+        <v>1299.12</v>
       </c>
       <c r="AE7" s="12" t="n">
-        <v>110.46</v>
+        <v>39.23</v>
       </c>
       <c r="AF7" s="12" t="n">
         <v>0</v>
@@ -18213,34 +18219,34 @@
     </row>
     <row r="8" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="n">
-        <v>309276</v>
+        <v>309346</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>97</v>
+        <v>68</v>
       </c>
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
       <c r="F8" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H8" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="G8" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="H8" s="9" t="s">
+      <c r="I8" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="J8" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="I8" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="J8" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="K8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>1299.12</v>
+        <v>2898.76</v>
       </c>
       <c r="M8" s="12" t="n">
         <v>0</v>
@@ -18249,55 +18255,55 @@
         <v>1</v>
       </c>
       <c r="O8" s="12" t="n">
-        <v>1299.12</v>
+        <v>2898.76</v>
       </c>
       <c r="P8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q8" s="13" t="n">
-        <v>0</v>
+        <v>0.004946</v>
       </c>
       <c r="R8" s="12" t="n">
-        <v>2</v>
+        <v>1.75</v>
       </c>
       <c r="S8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T8" s="14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="U8" s="15" t="s">
         <v>76</v>
       </c>
       <c r="V8" s="12" t="n">
-        <v>1367.5</v>
+        <v>2446.48</v>
       </c>
       <c r="W8" s="12" t="n">
-        <v>1.37</v>
+        <v>2.45</v>
       </c>
       <c r="X8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y8" s="12" t="n">
-        <v>12.31</v>
+        <v>22.02</v>
       </c>
       <c r="Z8" s="12" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="AA8" s="9" t="s">
         <v>77</v>
       </c>
       <c r="AB8" s="9" t="s">
-        <v>72</v>
+        <v>98</v>
       </c>
       <c r="AC8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AD8" s="12" t="n">
-        <v>1299.12</v>
+        <v>2898.76</v>
       </c>
       <c r="AE8" s="12" t="n">
-        <v>39.23</v>
+        <v>202.91</v>
       </c>
       <c r="AF8" s="12" t="n">
         <v>0</v>
@@ -18402,7 +18408,7 @@
         <v>81</v>
       </c>
       <c r="BN8" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="BO8" s="9" t="s">
         <v>79</v>
@@ -18416,10 +18422,10 @@
     </row>
     <row r="9" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="n">
-        <v>309346</v>
+        <v>309385</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
@@ -18428,13 +18434,13 @@
         <v>103</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="J9" s="9" t="s">
         <v>105</v>
@@ -18443,25 +18449,25 @@
         <v>74</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>2898.76</v>
+        <v>6597.51</v>
       </c>
       <c r="M9" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O9" s="12" t="n">
-        <v>2898.76</v>
+        <v>6011.4</v>
       </c>
       <c r="P9" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q9" s="13" t="n">
-        <v>0.004946</v>
+        <v>0</v>
       </c>
       <c r="R9" s="12" t="n">
-        <v>1.75</v>
+        <v>0</v>
       </c>
       <c r="S9" s="12" t="n">
         <v>0</v>
@@ -18473,34 +18479,34 @@
         <v>76</v>
       </c>
       <c r="V9" s="12" t="n">
-        <v>2446.48</v>
+        <v>5237.13</v>
       </c>
       <c r="W9" s="12" t="n">
-        <v>2.45</v>
+        <v>5.24</v>
       </c>
       <c r="X9" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y9" s="12" t="n">
-        <v>22.02</v>
+        <v>47.13</v>
       </c>
       <c r="Z9" s="12" t="n">
-        <v>28</v>
+        <v>57.33</v>
       </c>
       <c r="AA9" s="9" t="s">
         <v>77</v>
       </c>
       <c r="AB9" s="9" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="AC9" s="12" t="n">
-        <v>0</v>
+        <v>586.11</v>
       </c>
       <c r="AD9" s="12" t="n">
-        <v>2898.76</v>
+        <v>6011.4</v>
       </c>
       <c r="AE9" s="12" t="n">
-        <v>202.91</v>
+        <v>240.46</v>
       </c>
       <c r="AF9" s="12" t="n">
         <v>0</v>
@@ -18619,43 +18625,43 @@
     </row>
     <row r="10" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="n">
-        <v>309385</v>
+        <v>309395</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>68</v>
+        <v>108</v>
       </c>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
       <c r="F10" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>72</v>
+        <v>98</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="K10" s="11" t="s">
         <v>74</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>6597.51</v>
+        <v>3519.72</v>
       </c>
       <c r="M10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N10" s="12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O10" s="12" t="n">
-        <v>6011.4</v>
+        <v>3519.72</v>
       </c>
       <c r="P10" s="12" t="n">
         <v>0</v>
@@ -18670,40 +18676,40 @@
         <v>0</v>
       </c>
       <c r="T10" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U10" s="15" t="s">
         <v>76</v>
       </c>
       <c r="V10" s="12" t="n">
-        <v>5237.13</v>
+        <v>2970.54</v>
       </c>
       <c r="W10" s="12" t="n">
-        <v>5.24</v>
+        <v>2.97</v>
       </c>
       <c r="X10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y10" s="12" t="n">
-        <v>47.13</v>
+        <v>26.73</v>
       </c>
       <c r="Z10" s="12" t="n">
-        <v>57.33</v>
+        <v>28</v>
       </c>
       <c r="AA10" s="9" t="s">
         <v>77</v>
       </c>
       <c r="AB10" s="9" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="AC10" s="12" t="n">
-        <v>586.11</v>
+        <v>0</v>
       </c>
       <c r="AD10" s="12" t="n">
-        <v>6011.4</v>
+        <v>3519.72</v>
       </c>
       <c r="AE10" s="12" t="n">
-        <v>240.46</v>
+        <v>246.38</v>
       </c>
       <c r="AF10" s="12" t="n">
         <v>0</v>
@@ -18808,7 +18814,7 @@
         <v>81</v>
       </c>
       <c r="BN10" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BO10" s="9" t="s">
         <v>79</v>
@@ -18822,91 +18828,91 @@
     </row>
     <row r="11" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="n">
-        <v>309395</v>
+        <v>309398</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
       <c r="F11" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="K11" s="11" t="s">
         <v>74</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>3519.72</v>
+        <v>4157.93</v>
       </c>
       <c r="M11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O11" s="12" t="n">
-        <v>3519.72</v>
+        <v>4157.93</v>
       </c>
       <c r="P11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q11" s="13" t="n">
-        <v>0</v>
+        <v>0.004608</v>
       </c>
       <c r="R11" s="12" t="n">
-        <v>0</v>
+        <v>53.13</v>
       </c>
       <c r="S11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T11" s="14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="U11" s="15" t="s">
         <v>76</v>
       </c>
       <c r="V11" s="12" t="n">
-        <v>2970.54</v>
+        <v>3509.18</v>
       </c>
       <c r="W11" s="12" t="n">
-        <v>2.97</v>
+        <v>3.51</v>
       </c>
       <c r="X11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y11" s="12" t="n">
-        <v>26.73</v>
+        <v>31.58</v>
       </c>
       <c r="Z11" s="12" t="n">
-        <v>28</v>
+        <v>55.98</v>
       </c>
       <c r="AA11" s="9" t="s">
         <v>77</v>
       </c>
       <c r="AB11" s="9" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="AC11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AD11" s="12" t="n">
-        <v>3519.72</v>
+        <v>4157.93</v>
       </c>
       <c r="AE11" s="12" t="n">
-        <v>246.38</v>
+        <v>291.05</v>
       </c>
       <c r="AF11" s="12" t="n">
         <v>0</v>
@@ -19011,7 +19017,7 @@
         <v>81</v>
       </c>
       <c r="BN11" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="BO11" s="9" t="s">
         <v>79</v>
@@ -19025,91 +19031,91 @@
     </row>
     <row r="12" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="n">
-        <v>309398</v>
+        <v>309458</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
       <c r="F12" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="K12" s="11" t="s">
         <v>74</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>4157.93</v>
+        <v>960.97</v>
       </c>
       <c r="M12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N12" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O12" s="12" t="n">
-        <v>4157.93</v>
+        <v>875.6</v>
       </c>
       <c r="P12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" s="13" t="n">
-        <v>0.004608</v>
+        <v>0</v>
       </c>
       <c r="R12" s="12" t="n">
-        <v>53.13</v>
+        <v>0</v>
       </c>
       <c r="S12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T12" s="14" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="U12" s="15" t="s">
         <v>76</v>
       </c>
       <c r="V12" s="12" t="n">
-        <v>3509.18</v>
+        <v>0</v>
       </c>
       <c r="W12" s="12" t="n">
-        <v>3.51</v>
+        <v>0</v>
       </c>
       <c r="X12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y12" s="12" t="n">
-        <v>31.58</v>
+        <v>0</v>
       </c>
       <c r="Z12" s="12" t="n">
-        <v>55.98</v>
+        <v>28</v>
       </c>
       <c r="AA12" s="9" t="s">
         <v>77</v>
       </c>
       <c r="AB12" s="9" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="AC12" s="12" t="n">
-        <v>0</v>
+        <v>85.37</v>
       </c>
       <c r="AD12" s="12" t="n">
-        <v>4157.93</v>
+        <v>875.6</v>
       </c>
       <c r="AE12" s="12" t="n">
-        <v>291.05</v>
+        <v>61.29</v>
       </c>
       <c r="AF12" s="12" t="n">
         <v>0</v>
@@ -19118,7 +19124,7 @@
         <v>0</v>
       </c>
       <c r="AH12" s="12" t="n">
-        <v>0</v>
+        <v>89.72</v>
       </c>
       <c r="AI12" s="12" t="n">
         <v>0</v>
@@ -19199,25 +19205,25 @@
         <v>79</v>
       </c>
       <c r="BI12" s="14" t="s">
-        <v>79</v>
+        <v>123</v>
       </c>
       <c r="BJ12" s="9" t="s">
-        <v>79</v>
+        <v>124</v>
       </c>
       <c r="BK12" s="9" t="s">
-        <v>81</v>
+        <v>98</v>
       </c>
       <c r="BL12" s="14" t="s">
-        <v>79</v>
+        <v>125</v>
       </c>
       <c r="BM12" s="9" t="s">
-        <v>81</v>
+        <v>120</v>
       </c>
       <c r="BN12" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="BO12" s="9" t="s">
-        <v>79</v>
+        <v>127</v>
       </c>
       <c r="BP12" s="9" t="s">
         <v>79</v>
@@ -19228,34 +19234,34 @@
     </row>
     <row r="13" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="n">
-        <v>309458</v>
+        <v>309598</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
       <c r="F13" s="9" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>72</v>
+        <v>130</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="K13" s="11" t="s">
         <v>74</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>960.97</v>
+        <v>6432</v>
       </c>
       <c r="M13" s="12" t="n">
         <v>0</v>
@@ -19264,37 +19270,37 @@
         <v>1</v>
       </c>
       <c r="O13" s="12" t="n">
-        <v>875.6</v>
+        <v>6432</v>
       </c>
       <c r="P13" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q13" s="13" t="n">
-        <v>0</v>
+        <v>0.72</v>
       </c>
       <c r="R13" s="12" t="n">
-        <v>0</v>
+        <v>43.5</v>
       </c>
       <c r="S13" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T13" s="14" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="U13" s="15" t="s">
         <v>76</v>
       </c>
       <c r="V13" s="12" t="n">
-        <v>0</v>
+        <v>5949.34</v>
       </c>
       <c r="W13" s="12" t="n">
-        <v>0</v>
+        <v>5.95</v>
       </c>
       <c r="X13" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y13" s="12" t="n">
-        <v>0</v>
+        <v>53.54</v>
       </c>
       <c r="Z13" s="12" t="n">
         <v>28</v>
@@ -19303,16 +19309,16 @@
         <v>77</v>
       </c>
       <c r="AB13" s="9" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="AC13" s="12" t="n">
-        <v>85.37</v>
+        <v>0</v>
       </c>
       <c r="AD13" s="12" t="n">
-        <v>875.6</v>
+        <v>6432</v>
       </c>
       <c r="AE13" s="12" t="n">
-        <v>61.29</v>
+        <v>257.28</v>
       </c>
       <c r="AF13" s="12" t="n">
         <v>0</v>
@@ -19321,7 +19327,7 @@
         <v>0</v>
       </c>
       <c r="AH13" s="12" t="n">
-        <v>89.72</v>
+        <v>0</v>
       </c>
       <c r="AI13" s="12" t="n">
         <v>0</v>
@@ -19402,25 +19408,25 @@
         <v>79</v>
       </c>
       <c r="BI13" s="14" t="s">
-        <v>127</v>
+        <v>79</v>
       </c>
       <c r="BJ13" s="9" t="s">
-        <v>128</v>
+        <v>79</v>
       </c>
       <c r="BK13" s="9" t="s">
-        <v>104</v>
+        <v>81</v>
       </c>
       <c r="BL13" s="14" t="s">
-        <v>129</v>
+        <v>79</v>
       </c>
       <c r="BM13" s="9" t="s">
-        <v>124</v>
+        <v>81</v>
       </c>
       <c r="BN13" s="9" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="BO13" s="9" t="s">
-        <v>131</v>
+        <v>79</v>
       </c>
       <c r="BP13" s="9" t="s">
         <v>79</v>
@@ -19434,7 +19440,7 @@
     </row>
     <row r="15" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B15" s="17"/>
       <c r="C15" s="17"/>
@@ -19464,7 +19470,7 @@
     </row>
     <row r="16" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B16" s="18" t="s">
         <v>12</v>
@@ -19473,7 +19479,7 @@
         <v>15</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E16" s="18" t="s">
         <v>28</v>
@@ -19488,7 +19494,7 @@
         <v>31</v>
       </c>
       <c r="I16" s="18" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="J16" s="18" t="s">
         <v>33</v>
@@ -19500,7 +19506,7 @@
         <v>34</v>
       </c>
       <c r="M16" s="18" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="N16" s="18" t="s">
         <v>36</v>
@@ -19518,10 +19524,10 @@
         <v>16</v>
       </c>
       <c r="S16" s="18" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="T16" s="18" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="U16" s="18" t="s">
         <v>40</v>
@@ -19533,13 +19539,13 @@
         <v>21</v>
       </c>
       <c r="X16" s="18" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="Y16" s="18" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="Z16" s="18" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19556,13 +19562,13 @@
         <v>0</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>6282.49</v>
+        <v>825.33</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>81993.34</v>
+        <v>29695.13</v>
       </c>
       <c r="G17" s="19" t="n">
-        <v>3745.57</v>
+        <v>1653.64</v>
       </c>
       <c r="H17" s="19" t="n">
         <v>0</v>
@@ -19574,7 +19580,7 @@
         <v>89.72</v>
       </c>
       <c r="K17" s="19" t="n">
-        <v>88275.83</v>
+        <v>30520.46</v>
       </c>
       <c r="L17" s="19" t="n">
         <v>0</v>
@@ -19595,13 +19601,13 @@
         <v>0</v>
       </c>
       <c r="R17" s="20" t="n">
-        <v>0.539498</v>
+        <v>1.259498</v>
       </c>
       <c r="S17" s="19" t="n">
-        <v>81993.34</v>
+        <v>29695.13</v>
       </c>
       <c r="T17" s="19" t="n">
-        <v>88275.83</v>
+        <v>30520.46</v>
       </c>
       <c r="U17" s="19" t="n">
         <v>0</v>
@@ -19610,16 +19616,16 @@
         <v>0</v>
       </c>
       <c r="W17" s="19" t="n">
-        <v>70573.12</v>
+        <v>25356.71</v>
       </c>
       <c r="X17" s="19" t="n">
-        <v>70.59</v>
+        <v>25.37</v>
       </c>
       <c r="Y17" s="19" t="n">
         <v>0</v>
       </c>
       <c r="Z17" s="19" t="n">
-        <v>635.14</v>
+        <v>228.19</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19654,18 +19660,18 @@
         <v>49</v>
       </c>
       <c r="K18" s="18" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="L18" s="18" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="M18" s="18" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="n">
-        <v>61.56</v>
+        <v>102.56</v>
       </c>
       <c r="B19" s="19" t="n">
         <v>0</v>
@@ -19674,7 +19680,7 @@
         <v>0</v>
       </c>
       <c r="D19" s="19" t="n">
-        <v>73.05</v>
+        <v>38.63</v>
       </c>
       <c r="E19" s="19" t="n">
         <v>0</v>
@@ -19709,7 +19715,7 @@
     </row>
     <row r="21" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="21" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B21" s="21"/>
       <c r="C21" s="21"/>
@@ -19855,7 +19861,7 @@
     </row>
     <row r="23" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -19928,7 +19934,7 @@
     </row>
     <row r="24" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -20001,7 +20007,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -20147,7 +20153,7 @@
     </row>
     <row r="27" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -20220,7 +20226,7 @@
     </row>
     <row r="28" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -20293,7 +20299,7 @@
     </row>
     <row r="29" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -20366,7 +20372,7 @@
     </row>
     <row r="30" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -20439,7 +20445,7 @@
     </row>
     <row r="31" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>

</xml_diff>

<commit_message>
voucher correção+ atualização banco
</commit_message>
<xml_diff>
--- a/tratando_tabelas/finitura/entradas_finitura.xlsx
+++ b/tratando_tabelas/finitura/entradas_finitura.xlsx
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="154">
   <si>
     <t xml:space="preserve">Santri ADM 1.1.5.8 R1</t>
   </si>
   <si>
-    <t xml:space="preserve">Emitido em: 23/06/2026 04:30:38</t>
+    <t xml:space="preserve">Emitido em: 24/06/2026 07:16:26</t>
   </si>
   <si>
     <t xml:space="preserve">Relação de entradas - Sintético</t>
@@ -295,24 +295,6 @@
     <t xml:space="preserve">42260622670837000180550010000237991543419964</t>
   </si>
   <si>
-    <t xml:space="preserve">33.829 - STUDIO LAMPLUZ COMERCIO E SERVICOS LTDA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">585</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11/06/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11/07/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.299,12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35260658339477000186550010000005851000000592</t>
-  </si>
-  <si>
     <t xml:space="preserve">668.122</t>
   </si>
   <si>
@@ -376,36 +358,6 @@
     <t xml:space="preserve">42260675821546000102550100000022611710527158</t>
   </si>
   <si>
-    <t xml:space="preserve">9.974 - USINA DESIGN IND E COMERCIO DE ILUMINACAO LTDA-ME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10.156</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18/06/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14/07/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">960,97</t>
-  </si>
-  <si>
-    <t xml:space="preserve">401.449</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10.659 - RODO DANNY TRANSPORTES E LOGISTICAS EIRELI ME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">89,72</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35260610713221000160550020000101561000137024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35260611389565000200570050004014491000878201</t>
-  </si>
-  <si>
     <t xml:space="preserve">27.705 - DOKA - INDUSTRIA E COMERCIO LTDA</t>
   </si>
   <si>
@@ -422,6 +374,48 @@
   </si>
   <si>
     <t xml:space="preserve">42260601136190000131550010000639201764544670</t>
+  </si>
+  <si>
+    <t xml:space="preserve">672.196</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23/06/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.242,04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42260675339051000141550080006721961751051357</t>
+  </si>
+  <si>
+    <t xml:space="preserve">672.355</t>
+  </si>
+  <si>
+    <t xml:space="preserve">846,74</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42260675339051000141550080006723551288420762</t>
+  </si>
+  <si>
+    <t xml:space="preserve">672.686</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21/07/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.603,28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42260675339051000141550080006726861406105597</t>
+  </si>
+  <si>
+    <t xml:space="preserve">672.776</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.213,42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42260675339051000141550080006727761419936220</t>
   </si>
   <si>
     <t xml:space="preserve">Total geral</t>
@@ -17190,7 +17184,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:BQ31"/>
+  <dimension ref="A1:BQ33"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="18"/>
@@ -18016,34 +18010,34 @@
     </row>
     <row r="7" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="n">
-        <v>309276</v>
+        <v>309346</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
       <c r="F7" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H7" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="G7" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="H7" s="9" t="s">
+      <c r="I7" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="J7" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="J7" s="9" t="s">
-        <v>94</v>
       </c>
       <c r="K7" s="11" t="s">
         <v>74</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>1299.12</v>
+        <v>2898.76</v>
       </c>
       <c r="M7" s="12" t="n">
         <v>0</v>
@@ -18052,55 +18046,55 @@
         <v>1</v>
       </c>
       <c r="O7" s="12" t="n">
-        <v>1299.12</v>
+        <v>2898.76</v>
       </c>
       <c r="P7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q7" s="13" t="n">
-        <v>0</v>
+        <v>0.004946</v>
       </c>
       <c r="R7" s="12" t="n">
-        <v>2</v>
+        <v>1.75</v>
       </c>
       <c r="S7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T7" s="14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="U7" s="15" t="s">
         <v>76</v>
       </c>
       <c r="V7" s="12" t="n">
-        <v>1367.5</v>
+        <v>2446.48</v>
       </c>
       <c r="W7" s="12" t="n">
-        <v>1.37</v>
+        <v>2.45</v>
       </c>
       <c r="X7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y7" s="12" t="n">
-        <v>12.31</v>
+        <v>22.02</v>
       </c>
       <c r="Z7" s="12" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="AA7" s="9" t="s">
         <v>77</v>
       </c>
       <c r="AB7" s="9" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="AC7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AD7" s="12" t="n">
-        <v>1299.12</v>
+        <v>2898.76</v>
       </c>
       <c r="AE7" s="12" t="n">
-        <v>39.23</v>
+        <v>202.91</v>
       </c>
       <c r="AF7" s="12" t="n">
         <v>0</v>
@@ -18205,7 +18199,7 @@
         <v>81</v>
       </c>
       <c r="BN7" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="BO7" s="9" t="s">
         <v>79</v>
@@ -18219,10 +18213,10 @@
     </row>
     <row r="8" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="n">
-        <v>309346</v>
+        <v>309385</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
@@ -18231,13 +18225,13 @@
         <v>97</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>98</v>
+        <v>72</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="J8" s="9" t="s">
         <v>99</v>
@@ -18246,25 +18240,25 @@
         <v>74</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>2898.76</v>
+        <v>6597.51</v>
       </c>
       <c r="M8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O8" s="12" t="n">
-        <v>2898.76</v>
+        <v>6011.4</v>
       </c>
       <c r="P8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q8" s="13" t="n">
-        <v>0.004946</v>
+        <v>0</v>
       </c>
       <c r="R8" s="12" t="n">
-        <v>1.75</v>
+        <v>0</v>
       </c>
       <c r="S8" s="12" t="n">
         <v>0</v>
@@ -18276,34 +18270,34 @@
         <v>76</v>
       </c>
       <c r="V8" s="12" t="n">
-        <v>2446.48</v>
+        <v>5237.13</v>
       </c>
       <c r="W8" s="12" t="n">
-        <v>2.45</v>
+        <v>5.24</v>
       </c>
       <c r="X8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y8" s="12" t="n">
-        <v>22.02</v>
+        <v>47.13</v>
       </c>
       <c r="Z8" s="12" t="n">
-        <v>28</v>
+        <v>57.33</v>
       </c>
       <c r="AA8" s="9" t="s">
         <v>77</v>
       </c>
       <c r="AB8" s="9" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="AC8" s="12" t="n">
-        <v>0</v>
+        <v>586.11</v>
       </c>
       <c r="AD8" s="12" t="n">
-        <v>2898.76</v>
+        <v>6011.4</v>
       </c>
       <c r="AE8" s="12" t="n">
-        <v>202.91</v>
+        <v>240.46</v>
       </c>
       <c r="AF8" s="12" t="n">
         <v>0</v>
@@ -18422,7 +18416,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="n">
-        <v>309385</v>
+        <v>309395</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>102</v>
@@ -18437,28 +18431,28 @@
         <v>104</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="K9" s="11" t="s">
         <v>74</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>6597.51</v>
+        <v>3519.72</v>
       </c>
       <c r="M9" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O9" s="12" t="n">
-        <v>6011.4</v>
+        <v>3519.72</v>
       </c>
       <c r="P9" s="12" t="n">
         <v>0</v>
@@ -18473,40 +18467,40 @@
         <v>0</v>
       </c>
       <c r="T9" s="14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="U9" s="15" t="s">
         <v>76</v>
       </c>
       <c r="V9" s="12" t="n">
-        <v>5237.13</v>
+        <v>2970.54</v>
       </c>
       <c r="W9" s="12" t="n">
-        <v>5.24</v>
+        <v>2.97</v>
       </c>
       <c r="X9" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y9" s="12" t="n">
-        <v>47.13</v>
+        <v>26.73</v>
       </c>
       <c r="Z9" s="12" t="n">
-        <v>57.33</v>
+        <v>28</v>
       </c>
       <c r="AA9" s="9" t="s">
         <v>77</v>
       </c>
       <c r="AB9" s="9" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="AC9" s="12" t="n">
-        <v>586.11</v>
+        <v>0</v>
       </c>
       <c r="AD9" s="12" t="n">
-        <v>6011.4</v>
+        <v>3519.72</v>
       </c>
       <c r="AE9" s="12" t="n">
-        <v>240.46</v>
+        <v>246.38</v>
       </c>
       <c r="AF9" s="12" t="n">
         <v>0</v>
@@ -18611,7 +18605,7 @@
         <v>81</v>
       </c>
       <c r="BN9" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="BO9" s="9" t="s">
         <v>79</v>
@@ -18625,91 +18619,91 @@
     </row>
     <row r="10" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="n">
-        <v>309395</v>
+        <v>309398</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
       <c r="F10" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="G10" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="G10" s="10" t="s">
-        <v>110</v>
-      </c>
       <c r="H10" s="9" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="K10" s="11" t="s">
         <v>74</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>3519.72</v>
+        <v>4157.93</v>
       </c>
       <c r="M10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N10" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O10" s="12" t="n">
-        <v>3519.72</v>
+        <v>4157.93</v>
       </c>
       <c r="P10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q10" s="13" t="n">
-        <v>0</v>
+        <v>0.004608</v>
       </c>
       <c r="R10" s="12" t="n">
-        <v>0</v>
+        <v>53.13</v>
       </c>
       <c r="S10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T10" s="14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="U10" s="15" t="s">
         <v>76</v>
       </c>
       <c r="V10" s="12" t="n">
-        <v>2970.54</v>
+        <v>3509.18</v>
       </c>
       <c r="W10" s="12" t="n">
-        <v>2.97</v>
+        <v>3.51</v>
       </c>
       <c r="X10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y10" s="12" t="n">
-        <v>26.73</v>
+        <v>31.58</v>
       </c>
       <c r="Z10" s="12" t="n">
-        <v>28</v>
+        <v>55.98</v>
       </c>
       <c r="AA10" s="9" t="s">
         <v>77</v>
       </c>
       <c r="AB10" s="9" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="AC10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AD10" s="12" t="n">
-        <v>3519.72</v>
+        <v>4157.93</v>
       </c>
       <c r="AE10" s="12" t="n">
-        <v>246.38</v>
+        <v>291.05</v>
       </c>
       <c r="AF10" s="12" t="n">
         <v>0</v>
@@ -18814,7 +18808,7 @@
         <v>81</v>
       </c>
       <c r="BN10" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="BO10" s="9" t="s">
         <v>79</v>
@@ -18828,52 +18822,52 @@
     </row>
     <row r="11" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="n">
-        <v>309398</v>
+        <v>309598</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
       <c r="F11" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="H11" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="I11" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="J11" s="9" t="s">
         <v>115</v>
-      </c>
-      <c r="H11" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="I11" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="J11" s="9" t="s">
-        <v>99</v>
       </c>
       <c r="K11" s="11" t="s">
         <v>74</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>4157.93</v>
+        <v>6432</v>
       </c>
       <c r="M11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O11" s="12" t="n">
-        <v>4157.93</v>
+        <v>6432</v>
       </c>
       <c r="P11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q11" s="13" t="n">
-        <v>0.004608</v>
+        <v>0.72</v>
       </c>
       <c r="R11" s="12" t="n">
-        <v>53.13</v>
+        <v>43.5</v>
       </c>
       <c r="S11" s="12" t="n">
         <v>0</v>
@@ -18885,34 +18879,34 @@
         <v>76</v>
       </c>
       <c r="V11" s="12" t="n">
-        <v>3509.18</v>
+        <v>5949.34</v>
       </c>
       <c r="W11" s="12" t="n">
-        <v>3.51</v>
+        <v>5.95</v>
       </c>
       <c r="X11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y11" s="12" t="n">
-        <v>31.58</v>
+        <v>53.54</v>
       </c>
       <c r="Z11" s="12" t="n">
-        <v>55.98</v>
+        <v>28</v>
       </c>
       <c r="AA11" s="9" t="s">
         <v>77</v>
       </c>
       <c r="AB11" s="9" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="AC11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AD11" s="12" t="n">
-        <v>4157.93</v>
+        <v>6432</v>
       </c>
       <c r="AE11" s="12" t="n">
-        <v>291.05</v>
+        <v>257.28</v>
       </c>
       <c r="AF11" s="12" t="n">
         <v>0</v>
@@ -19031,34 +19025,34 @@
     </row>
     <row r="12" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="n">
-        <v>309458</v>
+        <v>309650</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>118</v>
+        <v>68</v>
       </c>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
       <c r="F12" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="I12" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="G12" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="I12" s="9" t="s">
-        <v>120</v>
-      </c>
       <c r="J12" s="9" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="K12" s="11" t="s">
         <v>74</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>960.97</v>
+        <v>9242.04</v>
       </c>
       <c r="M12" s="12" t="n">
         <v>0</v>
@@ -19067,37 +19061,37 @@
         <v>1</v>
       </c>
       <c r="O12" s="12" t="n">
-        <v>875.6</v>
+        <v>9242.04</v>
       </c>
       <c r="P12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" s="13" t="n">
-        <v>0</v>
+        <v>0.041862</v>
       </c>
       <c r="R12" s="12" t="n">
-        <v>0</v>
+        <v>14.04</v>
       </c>
       <c r="S12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T12" s="14" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="U12" s="15" t="s">
         <v>76</v>
       </c>
       <c r="V12" s="12" t="n">
-        <v>0</v>
+        <v>7800.06</v>
       </c>
       <c r="W12" s="12" t="n">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="X12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y12" s="12" t="n">
-        <v>0</v>
+        <v>70.2</v>
       </c>
       <c r="Z12" s="12" t="n">
         <v>28</v>
@@ -19106,16 +19100,16 @@
         <v>77</v>
       </c>
       <c r="AB12" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AC12" s="12" t="n">
-        <v>85.37</v>
+        <v>0</v>
       </c>
       <c r="AD12" s="12" t="n">
-        <v>875.6</v>
+        <v>9242.04</v>
       </c>
       <c r="AE12" s="12" t="n">
-        <v>61.29</v>
+        <v>646.94</v>
       </c>
       <c r="AF12" s="12" t="n">
         <v>0</v>
@@ -19124,7 +19118,7 @@
         <v>0</v>
       </c>
       <c r="AH12" s="12" t="n">
-        <v>89.72</v>
+        <v>0</v>
       </c>
       <c r="AI12" s="12" t="n">
         <v>0</v>
@@ -19205,25 +19199,25 @@
         <v>79</v>
       </c>
       <c r="BI12" s="14" t="s">
-        <v>123</v>
+        <v>79</v>
       </c>
       <c r="BJ12" s="9" t="s">
-        <v>124</v>
+        <v>79</v>
       </c>
       <c r="BK12" s="9" t="s">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="BL12" s="14" t="s">
-        <v>125</v>
+        <v>79</v>
       </c>
       <c r="BM12" s="9" t="s">
-        <v>120</v>
+        <v>81</v>
       </c>
       <c r="BN12" s="9" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="BO12" s="9" t="s">
-        <v>127</v>
+        <v>79</v>
       </c>
       <c r="BP12" s="9" t="s">
         <v>79</v>
@@ -19234,34 +19228,34 @@
     </row>
     <row r="13" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="n">
-        <v>309598</v>
+        <v>309669</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>128</v>
+        <v>68</v>
       </c>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
       <c r="F13" s="9" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="K13" s="11" t="s">
         <v>74</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>6432</v>
+        <v>846.74</v>
       </c>
       <c r="M13" s="12" t="n">
         <v>0</v>
@@ -19270,37 +19264,37 @@
         <v>1</v>
       </c>
       <c r="O13" s="12" t="n">
-        <v>6432</v>
+        <v>846.74</v>
       </c>
       <c r="P13" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q13" s="13" t="n">
-        <v>0.72</v>
+        <v>0</v>
       </c>
       <c r="R13" s="12" t="n">
-        <v>43.5</v>
+        <v>0.43</v>
       </c>
       <c r="S13" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T13" s="14" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="U13" s="15" t="s">
         <v>76</v>
       </c>
       <c r="V13" s="12" t="n">
-        <v>5949.34</v>
+        <v>714.62</v>
       </c>
       <c r="W13" s="12" t="n">
-        <v>5.95</v>
+        <v>0.71</v>
       </c>
       <c r="X13" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y13" s="12" t="n">
-        <v>53.54</v>
+        <v>6.43</v>
       </c>
       <c r="Z13" s="12" t="n">
         <v>28</v>
@@ -19309,16 +19303,16 @@
         <v>77</v>
       </c>
       <c r="AB13" s="9" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="AC13" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AD13" s="12" t="n">
-        <v>6432</v>
+        <v>846.74</v>
       </c>
       <c r="AE13" s="12" t="n">
-        <v>257.28</v>
+        <v>59.27</v>
       </c>
       <c r="AF13" s="12" t="n">
         <v>0</v>
@@ -19423,7 +19417,7 @@
         <v>81</v>
       </c>
       <c r="BN13" s="9" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="BO13" s="9" t="s">
         <v>79</v>
@@ -19436,242 +19430,527 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4"/>
+      <c r="A14" s="8" t="n">
+        <v>309673</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="J14" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="K14" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>2603.28</v>
+      </c>
+      <c r="M14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" s="12" t="n">
+        <v>2603.28</v>
+      </c>
+      <c r="P14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="13" t="n">
+        <v>0.00576</v>
+      </c>
+      <c r="R14" s="12" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="S14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="U14" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="V14" s="12" t="n">
+        <v>2197.11</v>
+      </c>
+      <c r="W14" s="12" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="X14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="12" t="n">
+        <v>19.77</v>
+      </c>
+      <c r="Z14" s="12" t="n">
+        <v>28</v>
+      </c>
+      <c r="AA14" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="AB14" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="AC14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD14" s="12" t="n">
+        <v>2603.28</v>
+      </c>
+      <c r="AE14" s="12" t="n">
+        <v>182.23</v>
+      </c>
+      <c r="AF14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL14" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AM14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN14" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AO14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ14" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AR14" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AS14" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="AT14" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AU14" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AV14" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AW14" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AX14" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AY14" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AZ14" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="BA14" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="BB14" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="BC14" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BD14" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BE14" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BF14" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BG14" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BH14" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BI14" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BJ14" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="BK14" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="BL14" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BM14" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="BN14" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BO14" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="BP14" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="BQ14" s="16" t="s">
+        <v>83</v>
+      </c>
     </row>
-    <row r="15" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17" t="s">
-        <v>134</v>
-      </c>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="17"/>
-      <c r="I15" s="17"/>
-      <c r="J15" s="17"/>
-      <c r="K15" s="17"/>
-      <c r="L15" s="17"/>
-      <c r="M15" s="17"/>
-      <c r="N15" s="17"/>
-      <c r="O15" s="17"/>
-      <c r="P15" s="17"/>
-      <c r="Q15" s="17"/>
-      <c r="R15" s="17"/>
-      <c r="S15" s="17"/>
-      <c r="T15" s="17"/>
-      <c r="U15" s="17"/>
-      <c r="V15" s="17"/>
-      <c r="W15" s="17"/>
-      <c r="X15" s="17"/>
-      <c r="Y15" s="17"/>
-      <c r="Z15" s="17"/>
+    <row r="15" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="n">
+        <v>309674</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="I15" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="J15" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="K15" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>2213.42</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" s="12" t="n">
+        <v>2213.42</v>
+      </c>
+      <c r="P15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="13" t="n">
+        <v>0.010353</v>
+      </c>
+      <c r="R15" s="12" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="S15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="U15" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="V15" s="12" t="n">
+        <v>1868.07</v>
+      </c>
+      <c r="W15" s="12" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="X15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="12" t="n">
+        <v>16.81</v>
+      </c>
+      <c r="Z15" s="12" t="n">
+        <v>28</v>
+      </c>
+      <c r="AA15" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="AB15" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="AC15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD15" s="12" t="n">
+        <v>2213.42</v>
+      </c>
+      <c r="AE15" s="12" t="n">
+        <v>154.94</v>
+      </c>
+      <c r="AF15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL15" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AM15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN15" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AO15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ15" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AR15" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AS15" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="AT15" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AU15" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AV15" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AW15" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AX15" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AY15" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AZ15" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="BA15" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="BB15" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="BC15" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BD15" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BE15" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BF15" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BG15" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BH15" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BI15" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BJ15" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="BK15" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="BL15" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="BM15" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="BN15" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="BO15" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="BP15" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="BQ15" s="16" t="s">
+        <v>83</v>
+      </c>
     </row>
-    <row r="16" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="s">
-        <v>135</v>
-      </c>
-      <c r="B16" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>136</v>
-      </c>
-      <c r="E16" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="F16" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="G16" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="H16" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="I16" s="18" t="s">
-        <v>137</v>
-      </c>
-      <c r="J16" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="K16" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="L16" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="M16" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="N16" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="O16" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="P16" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q16" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="R16" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="S16" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="T16" s="18" t="s">
-        <v>140</v>
-      </c>
-      <c r="U16" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="V16" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="W16" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="X16" s="18" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y16" s="18" t="s">
-        <v>142</v>
-      </c>
-      <c r="Z16" s="18" t="s">
-        <v>143</v>
-      </c>
+    <row r="16" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4"/>
     </row>
-    <row r="17" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="B17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="19" t="n">
-        <v>825.33</v>
-      </c>
-      <c r="F17" s="19" t="n">
-        <v>29695.13</v>
-      </c>
-      <c r="G17" s="19" t="n">
-        <v>1653.64</v>
-      </c>
-      <c r="H17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="19" t="n">
-        <v>89.72</v>
-      </c>
-      <c r="K17" s="19" t="n">
-        <v>30520.46</v>
-      </c>
-      <c r="L17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" s="20" t="n">
-        <v>1.259498</v>
-      </c>
-      <c r="S17" s="19" t="n">
-        <v>29695.13</v>
-      </c>
-      <c r="T17" s="19" t="n">
-        <v>30520.46</v>
-      </c>
-      <c r="U17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="V17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="W17" s="19" t="n">
-        <v>25356.71</v>
-      </c>
-      <c r="X17" s="19" t="n">
-        <v>25.37</v>
-      </c>
-      <c r="Y17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z17" s="19" t="n">
-        <v>228.19</v>
-      </c>
+    <row r="17" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
+      <c r="L17" s="17"/>
+      <c r="M17" s="17"/>
+      <c r="N17" s="17"/>
+      <c r="O17" s="17"/>
+      <c r="P17" s="17"/>
+      <c r="Q17" s="17"/>
+      <c r="R17" s="17"/>
+      <c r="S17" s="17"/>
+      <c r="T17" s="17"/>
+      <c r="U17" s="17"/>
+      <c r="V17" s="17"/>
+      <c r="W17" s="17"/>
+      <c r="X17" s="17"/>
+      <c r="Y17" s="17"/>
+      <c r="Z17" s="17"/>
     </row>
     <row r="18" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>17</v>
+        <v>133</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>25</v>
+        <v>134</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="H18" s="18" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="I18" s="18" t="s">
-        <v>48</v>
+        <v>135</v>
       </c>
       <c r="J18" s="18" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="K18" s="18" t="s">
-        <v>144</v>
+        <v>19</v>
       </c>
       <c r="L18" s="18" t="s">
-        <v>145</v>
+        <v>34</v>
       </c>
       <c r="M18" s="18" t="s">
-        <v>146</v>
+        <v>136</v>
+      </c>
+      <c r="N18" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="O18" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="P18" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q18" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="R18" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="S18" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="T18" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="U18" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="V18" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="W18" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="X18" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="Y18" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="Z18" s="18" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="n">
-        <v>102.56</v>
+        <v>11</v>
       </c>
       <c r="B19" s="19" t="n">
         <v>0</v>
@@ -19680,16 +19959,16 @@
         <v>0</v>
       </c>
       <c r="D19" s="19" t="n">
-        <v>38.63</v>
+        <v>0</v>
       </c>
       <c r="E19" s="19" t="n">
-        <v>0</v>
+        <v>739.96</v>
       </c>
       <c r="F19" s="19" t="n">
-        <v>0</v>
+        <v>42425.89</v>
       </c>
       <c r="G19" s="19" t="n">
-        <v>0</v>
+        <v>2596.5</v>
       </c>
       <c r="H19" s="19" t="n">
         <v>0</v>
@@ -19701,7 +19980,7 @@
         <v>0</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>0</v>
+        <v>43165.85</v>
       </c>
       <c r="L19" s="19" t="n">
         <v>0</v>
@@ -19709,232 +19988,207 @@
       <c r="M19" s="19" t="n">
         <v>0</v>
       </c>
+      <c r="N19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="20" t="n">
+        <v>1.317473</v>
+      </c>
+      <c r="S19" s="19" t="n">
+        <v>42425.89</v>
+      </c>
+      <c r="T19" s="19" t="n">
+        <v>43165.85</v>
+      </c>
+      <c r="U19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" s="19" t="n">
+        <v>36569.07</v>
+      </c>
+      <c r="X19" s="19" t="n">
+        <v>36.58</v>
+      </c>
+      <c r="Y19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="19" t="n">
+        <v>329.09</v>
+      </c>
     </row>
-    <row r="20" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4"/>
+    <row r="20" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="G20" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="H20" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="I20" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="J20" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="K20" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="L20" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="M20" s="18" t="s">
+        <v>144</v>
+      </c>
     </row>
-    <row r="21" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="s">
-        <v>147</v>
-      </c>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
-      <c r="H21" s="21"/>
-      <c r="I21" s="21"/>
-      <c r="J21" s="21"/>
-      <c r="K21" s="21"/>
-      <c r="L21" s="21"/>
-      <c r="M21" s="21"/>
-      <c r="N21" s="21"/>
-      <c r="O21" s="21"/>
-      <c r="P21" s="21"/>
-      <c r="Q21" s="21"/>
-      <c r="R21" s="21"/>
-      <c r="S21" s="21"/>
-      <c r="T21" s="21"/>
-      <c r="U21" s="21"/>
-      <c r="V21" s="21"/>
-      <c r="W21" s="21"/>
-      <c r="X21" s="21"/>
-      <c r="Y21" s="21"/>
-      <c r="Z21" s="21"/>
-      <c r="AA21" s="21"/>
-      <c r="AB21" s="21"/>
-      <c r="AC21" s="21"/>
-      <c r="AD21" s="21"/>
-      <c r="AE21" s="21"/>
-      <c r="AF21" s="21"/>
-      <c r="AG21" s="21"/>
-      <c r="AH21" s="21"/>
-      <c r="AI21" s="21"/>
-      <c r="AJ21" s="21"/>
-      <c r="AK21" s="21"/>
-      <c r="AL21" s="21"/>
-      <c r="AM21" s="21"/>
-      <c r="AN21" s="21"/>
-      <c r="AO21" s="21"/>
-      <c r="AP21" s="21"/>
-      <c r="AQ21" s="21"/>
-      <c r="AR21" s="21"/>
-      <c r="AS21" s="21"/>
-      <c r="AT21" s="21"/>
-      <c r="AU21" s="21"/>
-      <c r="AV21" s="21"/>
-      <c r="AW21" s="21"/>
-      <c r="AX21" s="21"/>
-      <c r="AY21" s="21"/>
-      <c r="AZ21" s="21"/>
-      <c r="BA21" s="21"/>
-      <c r="BB21" s="21"/>
-      <c r="BC21" s="21"/>
-      <c r="BD21" s="21"/>
-      <c r="BE21" s="21"/>
-      <c r="BF21" s="21"/>
-      <c r="BG21" s="21"/>
-      <c r="BH21" s="21"/>
-      <c r="BI21" s="21"/>
-      <c r="BJ21" s="21"/>
-      <c r="BK21" s="21"/>
-      <c r="BL21" s="21"/>
-      <c r="BM21" s="21"/>
-      <c r="BN21" s="21"/>
-      <c r="BO21" s="21"/>
-      <c r="BP21" s="21"/>
-      <c r="BQ21" s="21"/>
+    <row r="21" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="19" t="n">
+        <v>118.12</v>
+      </c>
+      <c r="B21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="19" t="n">
+        <v>35.46</v>
+      </c>
+      <c r="E21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
-      <c r="M22" s="4"/>
-      <c r="N22" s="4"/>
-      <c r="O22" s="4"/>
-      <c r="P22" s="4"/>
-      <c r="Q22" s="4"/>
-      <c r="R22" s="4"/>
-      <c r="S22" s="4"/>
-      <c r="T22" s="4"/>
-      <c r="U22" s="4"/>
-      <c r="V22" s="4"/>
-      <c r="W22" s="4"/>
-      <c r="X22" s="4"/>
-      <c r="Y22" s="4"/>
-      <c r="Z22" s="4"/>
-      <c r="AA22" s="4"/>
-      <c r="AB22" s="4"/>
-      <c r="AC22" s="4"/>
-      <c r="AD22" s="4"/>
-      <c r="AE22" s="4"/>
-      <c r="AF22" s="4"/>
-      <c r="AG22" s="4"/>
-      <c r="AH22" s="4"/>
-      <c r="AI22" s="4"/>
-      <c r="AJ22" s="4"/>
-      <c r="AK22" s="4"/>
-      <c r="AL22" s="4"/>
-      <c r="AM22" s="4"/>
-      <c r="AN22" s="4"/>
-      <c r="AO22" s="4"/>
-      <c r="AP22" s="4"/>
-      <c r="AQ22" s="4"/>
-      <c r="AR22" s="4"/>
-      <c r="AS22" s="4"/>
-      <c r="AT22" s="4"/>
-      <c r="AU22" s="4"/>
-      <c r="AV22" s="4"/>
-      <c r="AW22" s="4"/>
-      <c r="AX22" s="4"/>
-      <c r="AY22" s="4"/>
-      <c r="AZ22" s="4"/>
-      <c r="BA22" s="4"/>
-      <c r="BB22" s="4"/>
-      <c r="BC22" s="4"/>
-      <c r="BD22" s="4"/>
-      <c r="BE22" s="4"/>
-      <c r="BF22" s="4"/>
-      <c r="BG22" s="4"/>
-      <c r="BH22" s="4"/>
-      <c r="BI22" s="4"/>
-      <c r="BJ22" s="4"/>
-      <c r="BK22" s="4"/>
-      <c r="BL22" s="4"/>
-      <c r="BM22" s="4"/>
-      <c r="BN22" s="4"/>
-      <c r="BO22" s="4"/>
-      <c r="BP22" s="4"/>
-      <c r="BQ22" s="4"/>
+      <c r="A22" s="4"/>
     </row>
-    <row r="23" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
-      <c r="M23" s="4"/>
-      <c r="N23" s="4"/>
-      <c r="O23" s="4"/>
-      <c r="P23" s="4"/>
-      <c r="Q23" s="4"/>
-      <c r="R23" s="4"/>
-      <c r="S23" s="4"/>
-      <c r="T23" s="4"/>
-      <c r="U23" s="4"/>
-      <c r="V23" s="4"/>
-      <c r="W23" s="4"/>
-      <c r="X23" s="4"/>
-      <c r="Y23" s="4"/>
-      <c r="Z23" s="4"/>
-      <c r="AA23" s="4"/>
-      <c r="AB23" s="4"/>
-      <c r="AC23" s="4"/>
-      <c r="AD23" s="4"/>
-      <c r="AE23" s="4"/>
-      <c r="AF23" s="4"/>
-      <c r="AG23" s="4"/>
-      <c r="AH23" s="4"/>
-      <c r="AI23" s="4"/>
-      <c r="AJ23" s="4"/>
-      <c r="AK23" s="4"/>
-      <c r="AL23" s="4"/>
-      <c r="AM23" s="4"/>
-      <c r="AN23" s="4"/>
-      <c r="AO23" s="4"/>
-      <c r="AP23" s="4"/>
-      <c r="AQ23" s="4"/>
-      <c r="AR23" s="4"/>
-      <c r="AS23" s="4"/>
-      <c r="AT23" s="4"/>
-      <c r="AU23" s="4"/>
-      <c r="AV23" s="4"/>
-      <c r="AW23" s="4"/>
-      <c r="AX23" s="4"/>
-      <c r="AY23" s="4"/>
-      <c r="AZ23" s="4"/>
-      <c r="BA23" s="4"/>
-      <c r="BB23" s="4"/>
-      <c r="BC23" s="4"/>
-      <c r="BD23" s="4"/>
-      <c r="BE23" s="4"/>
-      <c r="BF23" s="4"/>
-      <c r="BG23" s="4"/>
-      <c r="BH23" s="4"/>
-      <c r="BI23" s="4"/>
-      <c r="BJ23" s="4"/>
-      <c r="BK23" s="4"/>
-      <c r="BL23" s="4"/>
-      <c r="BM23" s="4"/>
-      <c r="BN23" s="4"/>
-      <c r="BO23" s="4"/>
-      <c r="BP23" s="4"/>
-      <c r="BQ23" s="4"/>
+    <row r="23" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21" t="s">
+        <v>145</v>
+      </c>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="21"/>
+      <c r="H23" s="21"/>
+      <c r="I23" s="21"/>
+      <c r="J23" s="21"/>
+      <c r="K23" s="21"/>
+      <c r="L23" s="21"/>
+      <c r="M23" s="21"/>
+      <c r="N23" s="21"/>
+      <c r="O23" s="21"/>
+      <c r="P23" s="21"/>
+      <c r="Q23" s="21"/>
+      <c r="R23" s="21"/>
+      <c r="S23" s="21"/>
+      <c r="T23" s="21"/>
+      <c r="U23" s="21"/>
+      <c r="V23" s="21"/>
+      <c r="W23" s="21"/>
+      <c r="X23" s="21"/>
+      <c r="Y23" s="21"/>
+      <c r="Z23" s="21"/>
+      <c r="AA23" s="21"/>
+      <c r="AB23" s="21"/>
+      <c r="AC23" s="21"/>
+      <c r="AD23" s="21"/>
+      <c r="AE23" s="21"/>
+      <c r="AF23" s="21"/>
+      <c r="AG23" s="21"/>
+      <c r="AH23" s="21"/>
+      <c r="AI23" s="21"/>
+      <c r="AJ23" s="21"/>
+      <c r="AK23" s="21"/>
+      <c r="AL23" s="21"/>
+      <c r="AM23" s="21"/>
+      <c r="AN23" s="21"/>
+      <c r="AO23" s="21"/>
+      <c r="AP23" s="21"/>
+      <c r="AQ23" s="21"/>
+      <c r="AR23" s="21"/>
+      <c r="AS23" s="21"/>
+      <c r="AT23" s="21"/>
+      <c r="AU23" s="21"/>
+      <c r="AV23" s="21"/>
+      <c r="AW23" s="21"/>
+      <c r="AX23" s="21"/>
+      <c r="AY23" s="21"/>
+      <c r="AZ23" s="21"/>
+      <c r="BA23" s="21"/>
+      <c r="BB23" s="21"/>
+      <c r="BC23" s="21"/>
+      <c r="BD23" s="21"/>
+      <c r="BE23" s="21"/>
+      <c r="BF23" s="21"/>
+      <c r="BG23" s="21"/>
+      <c r="BH23" s="21"/>
+      <c r="BI23" s="21"/>
+      <c r="BJ23" s="21"/>
+      <c r="BK23" s="21"/>
+      <c r="BL23" s="21"/>
+      <c r="BM23" s="21"/>
+      <c r="BN23" s="21"/>
+      <c r="BO23" s="21"/>
+      <c r="BP23" s="21"/>
+      <c r="BQ23" s="21"/>
     </row>
     <row r="24" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>149</v>
+        <v>79</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -20007,7 +20261,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -20080,7 +20334,7 @@
     </row>
     <row r="26" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>26</v>
+        <v>147</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -20153,7 +20407,7 @@
     </row>
     <row r="27" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -20226,7 +20480,7 @@
     </row>
     <row r="28" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>152</v>
+        <v>26</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -20299,7 +20553,7 @@
     </row>
     <row r="29" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -20372,7 +20626,7 @@
     </row>
     <row r="30" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -20445,7 +20699,7 @@
     </row>
     <row r="31" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -20516,8 +20770,154 @@
       <c r="BP31" s="4"/>
       <c r="BQ31" s="4"/>
     </row>
+    <row r="32" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
+      <c r="I32" s="4"/>
+      <c r="J32" s="4"/>
+      <c r="K32" s="4"/>
+      <c r="L32" s="4"/>
+      <c r="M32" s="4"/>
+      <c r="N32" s="4"/>
+      <c r="O32" s="4"/>
+      <c r="P32" s="4"/>
+      <c r="Q32" s="4"/>
+      <c r="R32" s="4"/>
+      <c r="S32" s="4"/>
+      <c r="T32" s="4"/>
+      <c r="U32" s="4"/>
+      <c r="V32" s="4"/>
+      <c r="W32" s="4"/>
+      <c r="X32" s="4"/>
+      <c r="Y32" s="4"/>
+      <c r="Z32" s="4"/>
+      <c r="AA32" s="4"/>
+      <c r="AB32" s="4"/>
+      <c r="AC32" s="4"/>
+      <c r="AD32" s="4"/>
+      <c r="AE32" s="4"/>
+      <c r="AF32" s="4"/>
+      <c r="AG32" s="4"/>
+      <c r="AH32" s="4"/>
+      <c r="AI32" s="4"/>
+      <c r="AJ32" s="4"/>
+      <c r="AK32" s="4"/>
+      <c r="AL32" s="4"/>
+      <c r="AM32" s="4"/>
+      <c r="AN32" s="4"/>
+      <c r="AO32" s="4"/>
+      <c r="AP32" s="4"/>
+      <c r="AQ32" s="4"/>
+      <c r="AR32" s="4"/>
+      <c r="AS32" s="4"/>
+      <c r="AT32" s="4"/>
+      <c r="AU32" s="4"/>
+      <c r="AV32" s="4"/>
+      <c r="AW32" s="4"/>
+      <c r="AX32" s="4"/>
+      <c r="AY32" s="4"/>
+      <c r="AZ32" s="4"/>
+      <c r="BA32" s="4"/>
+      <c r="BB32" s="4"/>
+      <c r="BC32" s="4"/>
+      <c r="BD32" s="4"/>
+      <c r="BE32" s="4"/>
+      <c r="BF32" s="4"/>
+      <c r="BG32" s="4"/>
+      <c r="BH32" s="4"/>
+      <c r="BI32" s="4"/>
+      <c r="BJ32" s="4"/>
+      <c r="BK32" s="4"/>
+      <c r="BL32" s="4"/>
+      <c r="BM32" s="4"/>
+      <c r="BN32" s="4"/>
+      <c r="BO32" s="4"/>
+      <c r="BP32" s="4"/>
+      <c r="BQ32" s="4"/>
+    </row>
+    <row r="33" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="4"/>
+      <c r="K33" s="4"/>
+      <c r="L33" s="4"/>
+      <c r="M33" s="4"/>
+      <c r="N33" s="4"/>
+      <c r="O33" s="4"/>
+      <c r="P33" s="4"/>
+      <c r="Q33" s="4"/>
+      <c r="R33" s="4"/>
+      <c r="S33" s="4"/>
+      <c r="T33" s="4"/>
+      <c r="U33" s="4"/>
+      <c r="V33" s="4"/>
+      <c r="W33" s="4"/>
+      <c r="X33" s="4"/>
+      <c r="Y33" s="4"/>
+      <c r="Z33" s="4"/>
+      <c r="AA33" s="4"/>
+      <c r="AB33" s="4"/>
+      <c r="AC33" s="4"/>
+      <c r="AD33" s="4"/>
+      <c r="AE33" s="4"/>
+      <c r="AF33" s="4"/>
+      <c r="AG33" s="4"/>
+      <c r="AH33" s="4"/>
+      <c r="AI33" s="4"/>
+      <c r="AJ33" s="4"/>
+      <c r="AK33" s="4"/>
+      <c r="AL33" s="4"/>
+      <c r="AM33" s="4"/>
+      <c r="AN33" s="4"/>
+      <c r="AO33" s="4"/>
+      <c r="AP33" s="4"/>
+      <c r="AQ33" s="4"/>
+      <c r="AR33" s="4"/>
+      <c r="AS33" s="4"/>
+      <c r="AT33" s="4"/>
+      <c r="AU33" s="4"/>
+      <c r="AV33" s="4"/>
+      <c r="AW33" s="4"/>
+      <c r="AX33" s="4"/>
+      <c r="AY33" s="4"/>
+      <c r="AZ33" s="4"/>
+      <c r="BA33" s="4"/>
+      <c r="BB33" s="4"/>
+      <c r="BC33" s="4"/>
+      <c r="BD33" s="4"/>
+      <c r="BE33" s="4"/>
+      <c r="BF33" s="4"/>
+      <c r="BG33" s="4"/>
+      <c r="BH33" s="4"/>
+      <c r="BI33" s="4"/>
+      <c r="BJ33" s="4"/>
+      <c r="BK33" s="4"/>
+      <c r="BL33" s="4"/>
+      <c r="BM33" s="4"/>
+      <c r="BN33" s="4"/>
+      <c r="BO33" s="4"/>
+      <c r="BP33" s="4"/>
+      <c r="BQ33" s="4"/>
+    </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="27">
     <mergeCell ref="A1:BM1"/>
     <mergeCell ref="BN1:BQ1"/>
     <mergeCell ref="A2:BQ2"/>
@@ -20531,9 +20931,9 @@
     <mergeCell ref="B11:E11"/>
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="B13:E13"/>
-    <mergeCell ref="A15:Z15"/>
-    <mergeCell ref="A21:BQ21"/>
-    <mergeCell ref="A22:BQ22"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="A17:Z17"/>
     <mergeCell ref="A23:BQ23"/>
     <mergeCell ref="A24:BQ24"/>
     <mergeCell ref="A25:BQ25"/>
@@ -20543,6 +20943,8 @@
     <mergeCell ref="A29:BQ29"/>
     <mergeCell ref="A30:BQ30"/>
     <mergeCell ref="A31:BQ31"/>
+    <mergeCell ref="A32:BQ32"/>
+    <mergeCell ref="A33:BQ33"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
atualização banco + retirar botão
</commit_message>
<xml_diff>
--- a/tratando_tabelas/finitura/entradas_finitura.xlsx
+++ b/tratando_tabelas/finitura/entradas_finitura.xlsx
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="135">
   <si>
     <t xml:space="preserve">Santri ADM 1.1.5.8 R1</t>
   </si>
   <si>
-    <t xml:space="preserve">Emitido em: 25/06/2026 07:40:18</t>
+    <t xml:space="preserve">Emitido em: 26/06/2026 07:31:43</t>
   </si>
   <si>
     <t xml:space="preserve">Relação de entradas - Sintético</t>
@@ -226,28 +226,25 @@
     <t xml:space="preserve">Fornecedor substituto tributário</t>
   </si>
   <si>
-    <t xml:space="preserve">22.015 - FOCO METALLO FABRICACAO E MONTAGEM DE LUMINARIAS E COMERCIO</t>
+    <t xml:space="preserve">761 - DOCOL FV IND.E COM. DE METAIS SANITARIOS LTDA</t>
   </si>
   <si>
-    <t xml:space="preserve">23.799</t>
+    <t xml:space="preserve">668.122</t>
   </si>
   <si>
-    <t xml:space="preserve">1</t>
+    <t xml:space="preserve">8</t>
   </si>
   <si>
-    <t xml:space="preserve">15/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">16/06/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13/07/2026</t>
+    <t xml:space="preserve">15/07/2026</t>
   </si>
   <si>
     <t xml:space="preserve">XML</t>
   </si>
   <si>
-    <t xml:space="preserve">1.731,85</t>
+    <t xml:space="preserve">2.898,76</t>
   </si>
   <si>
     <t xml:space="preserve">Ag. chegada da mercadoria</t>
@@ -268,31 +265,10 @@
     <t xml:space="preserve">          </t>
   </si>
   <si>
-    <t xml:space="preserve">42260622670837000180550010000237991543419964</t>
+    <t xml:space="preserve">42260675339051000141550080006681221019457049</t>
   </si>
   <si>
     <t xml:space="preserve">Não</t>
-  </si>
-  <si>
-    <t xml:space="preserve">761 - DOCOL FV IND.E COM. DE METAIS SANITARIOS LTDA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">668.122</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17/06/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15/07/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.898,76</t>
-  </si>
-  <si>
-    <t xml:space="preserve">42260675339051000141550080006681221019457049</t>
   </si>
   <si>
     <t xml:space="preserve">16.008 - MEKAL METALURGICA KADOW S.A.</t>
@@ -310,25 +286,13 @@
     <t xml:space="preserve">35260657037392000180550030000104731553935734</t>
   </si>
   <si>
-    <t xml:space="preserve">3.101 - INDUSTRIA E COMERCIO DE MOLDURAS SANTA LUZIA LTDA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.261</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.157,93</t>
-  </si>
-  <si>
-    <t xml:space="preserve">42260675821546000102550100000022611710527158</t>
-  </si>
-  <si>
     <t xml:space="preserve">27.705 - DOKA - INDUSTRIA E COMERCIO LTDA</t>
   </si>
   <si>
     <t xml:space="preserve">63.920</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
   </si>
   <si>
     <t xml:space="preserve">22/06/2026</t>
@@ -385,25 +349,10 @@
     <t xml:space="preserve">42260675339051000141550080006727761419936220</t>
   </si>
   <si>
-    <t xml:space="preserve">9.974 - USINA DESIGN IND E COMERCIO DE ILUMINACAO LTDA-ME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10.377</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2</t>
+    <t xml:space="preserve">673.174</t>
   </si>
   <si>
     <t xml:space="preserve">24/06/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.263,37</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35260610713221000160550020000103771000140972</t>
-  </si>
-  <si>
-    <t xml:space="preserve">673.174</t>
   </si>
   <si>
     <t xml:space="preserve">2.764,74</t>
@@ -17178,7 +17127,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:BQ33"/>
+  <dimension ref="A1:BQ30"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="18"/>
@@ -17598,7 +17547,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="n">
-        <v>309242</v>
+        <v>309346</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>68</v>
@@ -17616,73 +17565,73 @@
         <v>71</v>
       </c>
       <c r="I5" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="J5" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="K5" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="K5" s="11" t="s">
-        <v>74</v>
-      </c>
       <c r="L5" s="12" t="n">
-        <v>1731.85</v>
+        <v>2898.76</v>
       </c>
       <c r="M5" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N5" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O5" s="12" t="n">
-        <v>1578</v>
+        <v>2898.76</v>
       </c>
       <c r="P5" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q5" s="13" t="n">
-        <v>0.5292</v>
+        <v>0.004946</v>
       </c>
       <c r="R5" s="12" t="n">
-        <v>0</v>
+        <v>1.75</v>
       </c>
       <c r="S5" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T5" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="U5" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="U5" s="15" t="s">
-        <v>76</v>
-      </c>
       <c r="V5" s="12" t="n">
-        <v>1409.94</v>
+        <v>2446.48</v>
       </c>
       <c r="W5" s="12" t="n">
-        <v>1.41</v>
+        <v>2.45</v>
       </c>
       <c r="X5" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y5" s="12" t="n">
-        <v>12.68</v>
+        <v>22.02</v>
       </c>
       <c r="Z5" s="12" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="AA5" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB5" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AC5" s="12" t="n">
-        <v>153.85</v>
+        <v>0</v>
       </c>
       <c r="AD5" s="12" t="n">
-        <v>1578</v>
+        <v>2898.76</v>
       </c>
       <c r="AE5" s="12" t="n">
-        <v>110.46</v>
+        <v>202.91</v>
       </c>
       <c r="AF5" s="12" t="n">
         <v>0</v>
@@ -17703,13 +17652,13 @@
         <v>0</v>
       </c>
       <c r="AL5" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AM5" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AN5" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AO5" s="12" t="n">
         <v>0</v>
@@ -17718,117 +17667,117 @@
         <v>0</v>
       </c>
       <c r="AQ5" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AR5" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AS5" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AR5" s="14" t="s">
+      <c r="AT5" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AU5" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AV5" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AW5" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AX5" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AY5" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AZ5" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BA5" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BB5" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="BC5" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AS5" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="AT5" s="14" t="s">
+      <c r="BD5" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AU5" s="14" t="s">
+      <c r="BE5" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AV5" s="14" t="s">
+      <c r="BF5" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AW5" s="14" t="s">
+      <c r="BG5" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AX5" s="14" t="s">
+      <c r="BH5" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AY5" s="14" t="s">
+      <c r="BI5" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AZ5" s="14" t="s">
+      <c r="BJ5" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="BA5" s="14" t="s">
+      <c r="BK5" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="BL5" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="BB5" s="10" t="s">
+      <c r="BM5" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="BC5" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BD5" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BE5" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF5" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BG5" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BH5" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BI5" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BJ5" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BK5" s="9" t="s">
+      <c r="BN5" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="BL5" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BM5" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="BN5" s="9" t="s">
+      <c r="BO5" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="BP5" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="BQ5" s="16" t="s">
         <v>82</v>
-      </c>
-      <c r="BO5" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BP5" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BQ5" s="16" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="n">
-        <v>309346</v>
+        <v>309395</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
       <c r="F6" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="G6" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="G6" s="10" t="s">
-        <v>86</v>
-      </c>
       <c r="H6" s="9" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>2898.76</v>
+        <v>3519.72</v>
       </c>
       <c r="M6" s="12" t="n">
         <v>0</v>
@@ -17837,55 +17786,55 @@
         <v>1</v>
       </c>
       <c r="O6" s="12" t="n">
-        <v>2898.76</v>
+        <v>3519.72</v>
       </c>
       <c r="P6" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q6" s="13" t="n">
-        <v>0.004946</v>
+        <v>0</v>
       </c>
       <c r="R6" s="12" t="n">
-        <v>1.75</v>
+        <v>0</v>
       </c>
       <c r="S6" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T6" s="14" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="U6" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="V6" s="12" t="n">
-        <v>2446.48</v>
+        <v>2970.54</v>
       </c>
       <c r="W6" s="12" t="n">
-        <v>2.45</v>
+        <v>2.97</v>
       </c>
       <c r="X6" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y6" s="12" t="n">
-        <v>22.02</v>
+        <v>26.73</v>
       </c>
       <c r="Z6" s="12" t="n">
         <v>28</v>
       </c>
       <c r="AA6" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB6" s="9" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="AC6" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AD6" s="12" t="n">
-        <v>2898.76</v>
+        <v>3519.72</v>
       </c>
       <c r="AE6" s="12" t="n">
-        <v>202.91</v>
+        <v>246.38</v>
       </c>
       <c r="AF6" s="12" t="n">
         <v>0</v>
@@ -17906,13 +17855,13 @@
         <v>0</v>
       </c>
       <c r="AL6" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AM6" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AN6" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AO6" s="12" t="n">
         <v>0</v>
@@ -17921,117 +17870,117 @@
         <v>0</v>
       </c>
       <c r="AQ6" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AR6" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AS6" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AR6" s="14" t="s">
+      <c r="AT6" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AU6" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AV6" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AW6" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AX6" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AY6" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AZ6" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BA6" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BB6" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="BC6" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AS6" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="AT6" s="14" t="s">
+      <c r="BD6" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AU6" s="14" t="s">
+      <c r="BE6" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AV6" s="14" t="s">
+      <c r="BF6" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AW6" s="14" t="s">
+      <c r="BG6" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AX6" s="14" t="s">
+      <c r="BH6" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AY6" s="14" t="s">
+      <c r="BI6" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AZ6" s="14" t="s">
+      <c r="BJ6" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="BA6" s="14" t="s">
+      <c r="BK6" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="BL6" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="BB6" s="10" t="s">
+      <c r="BM6" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="BC6" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BD6" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BE6" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF6" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BG6" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BH6" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BI6" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BJ6" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BK6" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="BL6" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BM6" s="9" t="s">
-        <v>81</v>
-      </c>
       <c r="BN6" s="9" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="BO6" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="BP6" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="BQ6" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="n">
-        <v>309395</v>
+        <v>309598</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
       <c r="F7" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="J7" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="G7" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="J7" s="9" t="s">
-        <v>88</v>
-      </c>
       <c r="K7" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>3519.72</v>
+        <v>6432</v>
       </c>
       <c r="M7" s="12" t="n">
         <v>0</v>
@@ -18040,55 +17989,55 @@
         <v>1</v>
       </c>
       <c r="O7" s="12" t="n">
-        <v>3519.72</v>
+        <v>6432</v>
       </c>
       <c r="P7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q7" s="13" t="n">
-        <v>0</v>
+        <v>0.72</v>
       </c>
       <c r="R7" s="12" t="n">
-        <v>0</v>
+        <v>43.5</v>
       </c>
       <c r="S7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T7" s="14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="U7" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="V7" s="12" t="n">
-        <v>2970.54</v>
+        <v>5949.34</v>
       </c>
       <c r="W7" s="12" t="n">
-        <v>2.97</v>
+        <v>5.95</v>
       </c>
       <c r="X7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y7" s="12" t="n">
-        <v>26.73</v>
+        <v>53.54</v>
       </c>
       <c r="Z7" s="12" t="n">
         <v>28</v>
       </c>
       <c r="AA7" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB7" s="9" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="AC7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AD7" s="12" t="n">
-        <v>3519.72</v>
+        <v>6432</v>
       </c>
       <c r="AE7" s="12" t="n">
-        <v>246.38</v>
+        <v>257.28</v>
       </c>
       <c r="AF7" s="12" t="n">
         <v>0</v>
@@ -18109,13 +18058,13 @@
         <v>0</v>
       </c>
       <c r="AL7" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AM7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AN7" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AO7" s="12" t="n">
         <v>0</v>
@@ -18124,174 +18073,174 @@
         <v>0</v>
       </c>
       <c r="AQ7" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AR7" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AS7" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AR7" s="14" t="s">
+      <c r="AT7" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AU7" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AV7" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AW7" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AX7" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AY7" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AZ7" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BA7" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BB7" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="BC7" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AS7" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="AT7" s="14" t="s">
+      <c r="BD7" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AU7" s="14" t="s">
+      <c r="BE7" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AV7" s="14" t="s">
+      <c r="BF7" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AW7" s="14" t="s">
+      <c r="BG7" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AX7" s="14" t="s">
+      <c r="BH7" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AY7" s="14" t="s">
+      <c r="BI7" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AZ7" s="14" t="s">
+      <c r="BJ7" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="BA7" s="14" t="s">
+      <c r="BK7" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="BL7" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="BB7" s="10" t="s">
+      <c r="BM7" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="BC7" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BD7" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BE7" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF7" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BG7" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BH7" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BI7" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BJ7" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BK7" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="BL7" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BM7" s="9" t="s">
-        <v>81</v>
-      </c>
       <c r="BN7" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="BO7" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="BP7" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="BQ7" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="n">
-        <v>309398</v>
+        <v>309650</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
       <c r="F8" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>98</v>
+        <v>70</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>4157.93</v>
+        <v>9242.04</v>
       </c>
       <c r="M8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O8" s="12" t="n">
-        <v>4157.93</v>
+        <v>9242.04</v>
       </c>
       <c r="P8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q8" s="13" t="n">
-        <v>0.004608</v>
+        <v>0.041862</v>
       </c>
       <c r="R8" s="12" t="n">
-        <v>53.13</v>
+        <v>14.04</v>
       </c>
       <c r="S8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T8" s="14" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="U8" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="V8" s="12" t="n">
-        <v>3509.18</v>
+        <v>7800.06</v>
       </c>
       <c r="W8" s="12" t="n">
-        <v>3.51</v>
+        <v>7.8</v>
       </c>
       <c r="X8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y8" s="12" t="n">
-        <v>31.58</v>
+        <v>70.2</v>
       </c>
       <c r="Z8" s="12" t="n">
-        <v>55.98</v>
+        <v>28</v>
       </c>
       <c r="AA8" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB8" s="9" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="AC8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AD8" s="12" t="n">
-        <v>4157.93</v>
+        <v>9242.04</v>
       </c>
       <c r="AE8" s="12" t="n">
-        <v>291.05</v>
+        <v>646.94</v>
       </c>
       <c r="AF8" s="12" t="n">
         <v>0</v>
@@ -18312,13 +18261,13 @@
         <v>0</v>
       </c>
       <c r="AL8" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AM8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AN8" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AO8" s="12" t="n">
         <v>0</v>
@@ -18327,117 +18276,117 @@
         <v>0</v>
       </c>
       <c r="AQ8" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AR8" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AS8" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AR8" s="14" t="s">
+      <c r="AT8" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AU8" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AV8" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AW8" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AX8" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AY8" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AZ8" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BA8" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BB8" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="BC8" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AS8" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="AT8" s="14" t="s">
+      <c r="BD8" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AU8" s="14" t="s">
+      <c r="BE8" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AV8" s="14" t="s">
+      <c r="BF8" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AW8" s="14" t="s">
+      <c r="BG8" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AX8" s="14" t="s">
+      <c r="BH8" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AY8" s="14" t="s">
+      <c r="BI8" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AZ8" s="14" t="s">
+      <c r="BJ8" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="BA8" s="14" t="s">
+      <c r="BK8" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="BL8" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="BB8" s="10" t="s">
+      <c r="BM8" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="BC8" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BD8" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BE8" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF8" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BG8" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BH8" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BI8" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BJ8" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BK8" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="BL8" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BM8" s="9" t="s">
-        <v>81</v>
-      </c>
       <c r="BN8" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="BO8" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="BP8" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="BQ8" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="n">
-        <v>309598</v>
+        <v>309669</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>101</v>
+        <v>68</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>70</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="K9" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>6432</v>
+        <v>846.74</v>
       </c>
       <c r="M9" s="12" t="n">
         <v>0</v>
@@ -18446,55 +18395,55 @@
         <v>1</v>
       </c>
       <c r="O9" s="12" t="n">
-        <v>6432</v>
+        <v>846.74</v>
       </c>
       <c r="P9" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q9" s="13" t="n">
-        <v>0.72</v>
+        <v>0</v>
       </c>
       <c r="R9" s="12" t="n">
-        <v>43.5</v>
+        <v>0.43</v>
       </c>
       <c r="S9" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T9" s="14" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="U9" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="V9" s="12" t="n">
-        <v>5949.34</v>
+        <v>714.62</v>
       </c>
       <c r="W9" s="12" t="n">
-        <v>5.95</v>
+        <v>0.71</v>
       </c>
       <c r="X9" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y9" s="12" t="n">
-        <v>53.54</v>
+        <v>6.43</v>
       </c>
       <c r="Z9" s="12" t="n">
         <v>28</v>
       </c>
       <c r="AA9" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB9" s="9" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="AC9" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AD9" s="12" t="n">
-        <v>6432</v>
+        <v>846.74</v>
       </c>
       <c r="AE9" s="12" t="n">
-        <v>257.28</v>
+        <v>59.27</v>
       </c>
       <c r="AF9" s="12" t="n">
         <v>0</v>
@@ -18515,13 +18464,13 @@
         <v>0</v>
       </c>
       <c r="AL9" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AM9" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AN9" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AO9" s="12" t="n">
         <v>0</v>
@@ -18530,117 +18479,117 @@
         <v>0</v>
       </c>
       <c r="AQ9" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AR9" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AS9" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AR9" s="14" t="s">
+      <c r="AT9" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AU9" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AV9" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AW9" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AX9" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AY9" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AZ9" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BA9" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BB9" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="BC9" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AS9" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="AT9" s="14" t="s">
+      <c r="BD9" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AU9" s="14" t="s">
+      <c r="BE9" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AV9" s="14" t="s">
+      <c r="BF9" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AW9" s="14" t="s">
+      <c r="BG9" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AX9" s="14" t="s">
+      <c r="BH9" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AY9" s="14" t="s">
+      <c r="BI9" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AZ9" s="14" t="s">
+      <c r="BJ9" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="BA9" s="14" t="s">
+      <c r="BK9" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="BL9" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="BB9" s="10" t="s">
+      <c r="BM9" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="BC9" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BD9" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BE9" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF9" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BG9" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BH9" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BI9" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BJ9" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BK9" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="BL9" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BM9" s="9" t="s">
-        <v>81</v>
-      </c>
       <c r="BN9" s="9" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="BO9" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="BP9" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="BQ9" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="n">
-        <v>309650</v>
+        <v>309673</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
       <c r="F10" s="9" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="H10" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="J10" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="I10" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="J10" s="9" t="s">
-        <v>104</v>
-      </c>
       <c r="K10" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>9242.04</v>
+        <v>2603.28</v>
       </c>
       <c r="M10" s="12" t="n">
         <v>0</v>
@@ -18649,55 +18598,55 @@
         <v>1</v>
       </c>
       <c r="O10" s="12" t="n">
-        <v>9242.04</v>
+        <v>2603.28</v>
       </c>
       <c r="P10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q10" s="13" t="n">
-        <v>0.041862</v>
+        <v>0.00576</v>
       </c>
       <c r="R10" s="12" t="n">
-        <v>14.04</v>
+        <v>1.44</v>
       </c>
       <c r="S10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T10" s="14" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="U10" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="V10" s="12" t="n">
-        <v>7800.06</v>
+        <v>2197.11</v>
       </c>
       <c r="W10" s="12" t="n">
-        <v>7.8</v>
+        <v>2.2</v>
       </c>
       <c r="X10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y10" s="12" t="n">
-        <v>70.2</v>
+        <v>19.77</v>
       </c>
       <c r="Z10" s="12" t="n">
         <v>28</v>
       </c>
       <c r="AA10" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB10" s="9" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="AC10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AD10" s="12" t="n">
-        <v>9242.04</v>
+        <v>2603.28</v>
       </c>
       <c r="AE10" s="12" t="n">
-        <v>646.94</v>
+        <v>182.23</v>
       </c>
       <c r="AF10" s="12" t="n">
         <v>0</v>
@@ -18718,13 +18667,13 @@
         <v>0</v>
       </c>
       <c r="AL10" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AM10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AN10" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AO10" s="12" t="n">
         <v>0</v>
@@ -18733,117 +18682,117 @@
         <v>0</v>
       </c>
       <c r="AQ10" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AR10" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AS10" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AR10" s="14" t="s">
+      <c r="AT10" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AU10" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AV10" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AW10" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AX10" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AY10" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AZ10" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BA10" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BB10" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="BC10" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AS10" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="AT10" s="14" t="s">
+      <c r="BD10" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AU10" s="14" t="s">
+      <c r="BE10" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AV10" s="14" t="s">
+      <c r="BF10" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AW10" s="14" t="s">
+      <c r="BG10" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AX10" s="14" t="s">
+      <c r="BH10" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AY10" s="14" t="s">
+      <c r="BI10" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AZ10" s="14" t="s">
+      <c r="BJ10" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="BA10" s="14" t="s">
+      <c r="BK10" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="BL10" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="BB10" s="10" t="s">
+      <c r="BM10" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="BC10" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BD10" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BE10" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF10" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BG10" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BH10" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BI10" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BJ10" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BK10" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="BL10" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BM10" s="9" t="s">
-        <v>81</v>
-      </c>
       <c r="BN10" s="9" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="BO10" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="BP10" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="BQ10" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="n">
-        <v>309669</v>
+        <v>309674</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
       <c r="F11" s="9" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="H11" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="I11" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="J11" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="I11" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="J11" s="9" t="s">
-        <v>104</v>
-      </c>
       <c r="K11" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>846.74</v>
+        <v>2213.42</v>
       </c>
       <c r="M11" s="12" t="n">
         <v>0</v>
@@ -18852,55 +18801,55 @@
         <v>1</v>
       </c>
       <c r="O11" s="12" t="n">
-        <v>846.74</v>
+        <v>2213.42</v>
       </c>
       <c r="P11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q11" s="13" t="n">
-        <v>0</v>
+        <v>0.010353</v>
       </c>
       <c r="R11" s="12" t="n">
-        <v>0.43</v>
+        <v>1.65</v>
       </c>
       <c r="S11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T11" s="14" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="U11" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="V11" s="12" t="n">
-        <v>714.62</v>
+        <v>1868.07</v>
       </c>
       <c r="W11" s="12" t="n">
-        <v>0.71</v>
+        <v>1.87</v>
       </c>
       <c r="X11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y11" s="12" t="n">
-        <v>6.43</v>
+        <v>16.81</v>
       </c>
       <c r="Z11" s="12" t="n">
         <v>28</v>
       </c>
       <c r="AA11" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB11" s="9" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="AC11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AD11" s="12" t="n">
-        <v>846.74</v>
+        <v>2213.42</v>
       </c>
       <c r="AE11" s="12" t="n">
-        <v>59.27</v>
+        <v>154.94</v>
       </c>
       <c r="AF11" s="12" t="n">
         <v>0</v>
@@ -18921,13 +18870,13 @@
         <v>0</v>
       </c>
       <c r="AL11" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AM11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AN11" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AO11" s="12" t="n">
         <v>0</v>
@@ -18936,174 +18885,174 @@
         <v>0</v>
       </c>
       <c r="AQ11" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AR11" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AS11" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AR11" s="14" t="s">
+      <c r="AT11" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AU11" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AV11" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AW11" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AX11" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AY11" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AZ11" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BA11" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BB11" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="BC11" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AS11" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="AT11" s="14" t="s">
+      <c r="BD11" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AU11" s="14" t="s">
+      <c r="BE11" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AV11" s="14" t="s">
+      <c r="BF11" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AW11" s="14" t="s">
+      <c r="BG11" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AX11" s="14" t="s">
+      <c r="BH11" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AY11" s="14" t="s">
+      <c r="BI11" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AZ11" s="14" t="s">
+      <c r="BJ11" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="BA11" s="14" t="s">
+      <c r="BK11" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="BL11" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="BB11" s="10" t="s">
+      <c r="BM11" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="BC11" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BD11" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BE11" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF11" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BG11" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BH11" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BI11" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BJ11" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BK11" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="BL11" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BM11" s="9" t="s">
-        <v>81</v>
-      </c>
       <c r="BN11" s="9" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="BO11" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="BP11" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="BQ11" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="n">
-        <v>309673</v>
+        <v>309734</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
       <c r="F12" s="9" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="K12" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>2603.28</v>
+        <v>2764.74</v>
       </c>
       <c r="M12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="N12" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O12" s="12" t="n">
-        <v>2603.28</v>
+        <v>2638.8</v>
       </c>
       <c r="P12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" s="13" t="n">
-        <v>0.00576</v>
+        <v>0.035898</v>
       </c>
       <c r="R12" s="12" t="n">
-        <v>1.44</v>
+        <v>4.91</v>
       </c>
       <c r="S12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="T12" s="14" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="U12" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="V12" s="12" t="n">
-        <v>2197.11</v>
+        <v>2227.08</v>
       </c>
       <c r="W12" s="12" t="n">
-        <v>2.2</v>
+        <v>2.23</v>
       </c>
       <c r="X12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="Y12" s="12" t="n">
-        <v>19.77</v>
+        <v>20.04</v>
       </c>
       <c r="Z12" s="12" t="n">
         <v>28</v>
       </c>
       <c r="AA12" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AB12" s="9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="AC12" s="12" t="n">
-        <v>0</v>
+        <v>125.94</v>
       </c>
       <c r="AD12" s="12" t="n">
-        <v>2603.28</v>
+        <v>2638.8</v>
       </c>
       <c r="AE12" s="12" t="n">
-        <v>182.23</v>
+        <v>184.72</v>
       </c>
       <c r="AF12" s="12" t="n">
         <v>0</v>
@@ -19124,13 +19073,13 @@
         <v>0</v>
       </c>
       <c r="AL12" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AM12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AN12" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AO12" s="12" t="n">
         <v>0</v>
@@ -19139,1050 +19088,660 @@
         <v>0</v>
       </c>
       <c r="AQ12" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AR12" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AS12" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AR12" s="14" t="s">
+      <c r="AT12" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AU12" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AV12" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AW12" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AX12" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AY12" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="AZ12" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BA12" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="BB12" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="BC12" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AS12" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="AT12" s="14" t="s">
+      <c r="BD12" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AU12" s="14" t="s">
+      <c r="BE12" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AV12" s="14" t="s">
+      <c r="BF12" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AW12" s="14" t="s">
+      <c r="BG12" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AX12" s="14" t="s">
+      <c r="BH12" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AY12" s="14" t="s">
+      <c r="BI12" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="AZ12" s="14" t="s">
+      <c r="BJ12" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="BA12" s="14" t="s">
+      <c r="BK12" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="BL12" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="BB12" s="10" t="s">
+      <c r="BM12" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="BC12" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BD12" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BE12" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF12" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BG12" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BH12" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BI12" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BJ12" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BK12" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="BL12" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BM12" s="9" t="s">
-        <v>81</v>
-      </c>
       <c r="BN12" s="9" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="BO12" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="BP12" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="BQ12" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="n">
-        <v>309674</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9" t="s">
+      <c r="A13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="17" t="s">
+        <v>113</v>
+      </c>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="17"/>
+      <c r="M14" s="17"/>
+      <c r="N14" s="17"/>
+      <c r="O14" s="17"/>
+      <c r="P14" s="17"/>
+      <c r="Q14" s="17"/>
+      <c r="R14" s="17"/>
+      <c r="S14" s="17"/>
+      <c r="T14" s="17"/>
+      <c r="U14" s="17"/>
+      <c r="V14" s="17"/>
+      <c r="W14" s="17"/>
+      <c r="X14" s="17"/>
+      <c r="Y14" s="17"/>
+      <c r="Z14" s="17"/>
+    </row>
+    <row r="15" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G15" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="H15" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="I15" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="J15" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="K15" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="L15" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="M15" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="N15" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="O15" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="P15" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q15" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="R15" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="S15" s="18" t="s">
         <v>118</v>
       </c>
-      <c r="G13" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="H13" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="I13" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="J13" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="K13" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="L13" s="12" t="n">
-        <v>2213.42</v>
-      </c>
-      <c r="M13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="O13" s="12" t="n">
-        <v>2213.42</v>
-      </c>
-      <c r="P13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="13" t="n">
-        <v>0.010353</v>
-      </c>
-      <c r="R13" s="12" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="S13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" s="14" t="s">
+      <c r="T15" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="U13" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="V13" s="12" t="n">
-        <v>1868.07</v>
-      </c>
-      <c r="W13" s="12" t="n">
-        <v>1.87</v>
-      </c>
-      <c r="X13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y13" s="12" t="n">
-        <v>16.81</v>
-      </c>
-      <c r="Z13" s="12" t="n">
-        <v>28</v>
-      </c>
-      <c r="AA13" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="AB13" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="AC13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD13" s="12" t="n">
-        <v>2213.42</v>
-      </c>
-      <c r="AE13" s="12" t="n">
-        <v>154.94</v>
-      </c>
-      <c r="AF13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL13" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AM13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN13" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AO13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ13" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AR13" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AS13" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="AT13" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AU13" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AV13" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AW13" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AX13" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AY13" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AZ13" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="BA13" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="BB13" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="BC13" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BD13" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BE13" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF13" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BG13" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BH13" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BI13" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BJ13" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BK13" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="BL13" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BM13" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="BN13" s="9" t="s">
+      <c r="U15" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="V15" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="W15" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="X15" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="BO13" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BP13" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BQ13" s="16" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="n">
-        <v>309723</v>
-      </c>
-      <c r="B14" s="9" t="s">
+      <c r="Y15" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9" t="s">
+      <c r="Z15" s="18" t="s">
         <v>122</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="I14" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="J14" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="K14" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="L14" s="12" t="n">
-        <v>1263.37</v>
-      </c>
-      <c r="M14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="O14" s="12" t="n">
-        <v>1151.14</v>
-      </c>
-      <c r="P14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="U14" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="V14" s="12" t="n">
-        <v>971.54</v>
-      </c>
-      <c r="W14" s="12" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="X14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y14" s="12" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="Z14" s="12" t="n">
-        <v>28</v>
-      </c>
-      <c r="AA14" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="AB14" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="AC14" s="12" t="n">
-        <v>112.23</v>
-      </c>
-      <c r="AD14" s="12" t="n">
-        <v>1151.14</v>
-      </c>
-      <c r="AE14" s="12" t="n">
-        <v>80.58</v>
-      </c>
-      <c r="AF14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL14" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AM14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN14" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AO14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ14" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AR14" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AS14" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="AT14" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AU14" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AV14" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AW14" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AX14" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AY14" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AZ14" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="BA14" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="BB14" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="BC14" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BD14" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BE14" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF14" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BG14" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BH14" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BI14" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BJ14" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BK14" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="BL14" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BM14" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="BN14" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="BO14" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BP14" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BQ14" s="16" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="n">
-        <v>309734</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="H15" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="I15" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="J15" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="K15" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>2764.74</v>
-      </c>
-      <c r="M15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="O15" s="12" t="n">
-        <v>2638.8</v>
-      </c>
-      <c r="P15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="13" t="n">
-        <v>0.035898</v>
-      </c>
-      <c r="R15" s="12" t="n">
-        <v>4.91</v>
-      </c>
-      <c r="S15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T15" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="U15" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="V15" s="12" t="n">
-        <v>2227.08</v>
-      </c>
-      <c r="W15" s="12" t="n">
-        <v>2.23</v>
-      </c>
-      <c r="X15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y15" s="12" t="n">
-        <v>20.04</v>
-      </c>
-      <c r="Z15" s="12" t="n">
-        <v>28</v>
-      </c>
-      <c r="AA15" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="AB15" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="AC15" s="12" t="n">
-        <v>125.94</v>
-      </c>
-      <c r="AD15" s="12" t="n">
-        <v>2638.8</v>
-      </c>
-      <c r="AE15" s="12" t="n">
-        <v>184.72</v>
-      </c>
-      <c r="AF15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL15" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AM15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN15" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AO15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP15" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ15" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AR15" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AS15" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="AT15" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AU15" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AV15" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AW15" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AX15" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AY15" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="AZ15" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="BA15" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="BB15" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="BC15" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BD15" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BE15" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BF15" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BG15" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BH15" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BI15" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BJ15" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BK15" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="BL15" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="BM15" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="BN15" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="BO15" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BP15" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="BQ15" s="16" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4"/>
+      <c r="A16" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="19" t="n">
+        <v>125.94</v>
+      </c>
+      <c r="F16" s="19" t="n">
+        <v>30394.76</v>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>1934.67</v>
+      </c>
+      <c r="H16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="19" t="n">
+        <v>30520.7</v>
+      </c>
+      <c r="L16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="20" t="n">
+        <v>0.818819</v>
+      </c>
+      <c r="S16" s="19" t="n">
+        <v>30394.76</v>
+      </c>
+      <c r="T16" s="19" t="n">
+        <v>30520.7</v>
+      </c>
+      <c r="U16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" s="19" t="n">
+        <v>26173.3</v>
+      </c>
+      <c r="X16" s="19" t="n">
+        <v>26.18</v>
+      </c>
+      <c r="Y16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" s="19" t="n">
+        <v>235.54</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
-        <v>130</v>
-      </c>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="17"/>
-      <c r="L17" s="17"/>
-      <c r="M17" s="17"/>
-      <c r="N17" s="17"/>
-      <c r="O17" s="17"/>
-      <c r="P17" s="17"/>
-      <c r="Q17" s="17"/>
-      <c r="R17" s="17"/>
-      <c r="S17" s="17"/>
-      <c r="T17" s="17"/>
-      <c r="U17" s="17"/>
-      <c r="V17" s="17"/>
-      <c r="W17" s="17"/>
-      <c r="X17" s="17"/>
-      <c r="Y17" s="17"/>
-      <c r="Z17" s="17"/>
+      <c r="A17" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="F17" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="G17" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="H17" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="I17" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="J17" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="K17" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="L17" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="M17" s="18" t="s">
+        <v>125</v>
+      </c>
     </row>
-    <row r="18" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
-        <v>131</v>
-      </c>
-      <c r="B18" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="D18" s="18" t="s">
-        <v>132</v>
-      </c>
-      <c r="E18" s="18" t="s">
+    <row r="18" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="19" t="n">
+        <v>67.72</v>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="19" t="n">
         <v>28</v>
       </c>
-      <c r="F18" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="G18" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="H18" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="I18" s="18" t="s">
-        <v>133</v>
-      </c>
-      <c r="J18" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="K18" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="L18" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="M18" s="18" t="s">
-        <v>134</v>
-      </c>
-      <c r="N18" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="O18" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="P18" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q18" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="R18" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="S18" s="18" t="s">
-        <v>135</v>
-      </c>
-      <c r="T18" s="18" t="s">
-        <v>136</v>
-      </c>
-      <c r="U18" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="V18" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="W18" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="X18" s="18" t="s">
-        <v>137</v>
-      </c>
-      <c r="Y18" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="Z18" s="18" t="s">
-        <v>139</v>
+      <c r="E18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="B19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="19" t="n">
-        <v>392.02</v>
-      </c>
-      <c r="F19" s="19" t="n">
-        <v>37281.83</v>
-      </c>
-      <c r="G19" s="19" t="n">
-        <v>2416.76</v>
-      </c>
-      <c r="H19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" s="19" t="n">
-        <v>37673.85</v>
-      </c>
-      <c r="L19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" s="20" t="n">
-        <v>1.352627</v>
-      </c>
-      <c r="S19" s="19" t="n">
-        <v>37281.83</v>
-      </c>
-      <c r="T19" s="19" t="n">
-        <v>37673.85</v>
-      </c>
-      <c r="U19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="V19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="W19" s="19" t="n">
-        <v>32063.96</v>
-      </c>
-      <c r="X19" s="19" t="n">
-        <v>32.08</v>
-      </c>
-      <c r="Y19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z19" s="19" t="n">
-        <v>288.55</v>
-      </c>
+      <c r="A19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="B20" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="C20" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="D20" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="E20" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G20" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="H20" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="I20" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="J20" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="K20" s="18" t="s">
-        <v>140</v>
-      </c>
-      <c r="L20" s="18" t="s">
-        <v>141</v>
-      </c>
-      <c r="M20" s="18" t="s">
-        <v>142</v>
-      </c>
+      <c r="A20" s="21" t="s">
+        <v>126</v>
+      </c>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="21"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="21"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="21"/>
+      <c r="L20" s="21"/>
+      <c r="M20" s="21"/>
+      <c r="N20" s="21"/>
+      <c r="O20" s="21"/>
+      <c r="P20" s="21"/>
+      <c r="Q20" s="21"/>
+      <c r="R20" s="21"/>
+      <c r="S20" s="21"/>
+      <c r="T20" s="21"/>
+      <c r="U20" s="21"/>
+      <c r="V20" s="21"/>
+      <c r="W20" s="21"/>
+      <c r="X20" s="21"/>
+      <c r="Y20" s="21"/>
+      <c r="Z20" s="21"/>
+      <c r="AA20" s="21"/>
+      <c r="AB20" s="21"/>
+      <c r="AC20" s="21"/>
+      <c r="AD20" s="21"/>
+      <c r="AE20" s="21"/>
+      <c r="AF20" s="21"/>
+      <c r="AG20" s="21"/>
+      <c r="AH20" s="21"/>
+      <c r="AI20" s="21"/>
+      <c r="AJ20" s="21"/>
+      <c r="AK20" s="21"/>
+      <c r="AL20" s="21"/>
+      <c r="AM20" s="21"/>
+      <c r="AN20" s="21"/>
+      <c r="AO20" s="21"/>
+      <c r="AP20" s="21"/>
+      <c r="AQ20" s="21"/>
+      <c r="AR20" s="21"/>
+      <c r="AS20" s="21"/>
+      <c r="AT20" s="21"/>
+      <c r="AU20" s="21"/>
+      <c r="AV20" s="21"/>
+      <c r="AW20" s="21"/>
+      <c r="AX20" s="21"/>
+      <c r="AY20" s="21"/>
+      <c r="AZ20" s="21"/>
+      <c r="BA20" s="21"/>
+      <c r="BB20" s="21"/>
+      <c r="BC20" s="21"/>
+      <c r="BD20" s="21"/>
+      <c r="BE20" s="21"/>
+      <c r="BF20" s="21"/>
+      <c r="BG20" s="21"/>
+      <c r="BH20" s="21"/>
+      <c r="BI20" s="21"/>
+      <c r="BJ20" s="21"/>
+      <c r="BK20" s="21"/>
+      <c r="BL20" s="21"/>
+      <c r="BM20" s="21"/>
+      <c r="BN20" s="21"/>
+      <c r="BO20" s="21"/>
+      <c r="BP20" s="21"/>
+      <c r="BQ20" s="21"/>
     </row>
     <row r="21" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="n">
-        <v>120.85</v>
-      </c>
-      <c r="B21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="19" t="n">
-        <v>31.41</v>
-      </c>
-      <c r="E21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" s="19" t="n">
-        <v>0</v>
-      </c>
+      <c r="A21" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4"/>
+      <c r="O21" s="4"/>
+      <c r="P21" s="4"/>
+      <c r="Q21" s="4"/>
+      <c r="R21" s="4"/>
+      <c r="S21" s="4"/>
+      <c r="T21" s="4"/>
+      <c r="U21" s="4"/>
+      <c r="V21" s="4"/>
+      <c r="W21" s="4"/>
+      <c r="X21" s="4"/>
+      <c r="Y21" s="4"/>
+      <c r="Z21" s="4"/>
+      <c r="AA21" s="4"/>
+      <c r="AB21" s="4"/>
+      <c r="AC21" s="4"/>
+      <c r="AD21" s="4"/>
+      <c r="AE21" s="4"/>
+      <c r="AF21" s="4"/>
+      <c r="AG21" s="4"/>
+      <c r="AH21" s="4"/>
+      <c r="AI21" s="4"/>
+      <c r="AJ21" s="4"/>
+      <c r="AK21" s="4"/>
+      <c r="AL21" s="4"/>
+      <c r="AM21" s="4"/>
+      <c r="AN21" s="4"/>
+      <c r="AO21" s="4"/>
+      <c r="AP21" s="4"/>
+      <c r="AQ21" s="4"/>
+      <c r="AR21" s="4"/>
+      <c r="AS21" s="4"/>
+      <c r="AT21" s="4"/>
+      <c r="AU21" s="4"/>
+      <c r="AV21" s="4"/>
+      <c r="AW21" s="4"/>
+      <c r="AX21" s="4"/>
+      <c r="AY21" s="4"/>
+      <c r="AZ21" s="4"/>
+      <c r="BA21" s="4"/>
+      <c r="BB21" s="4"/>
+      <c r="BC21" s="4"/>
+      <c r="BD21" s="4"/>
+      <c r="BE21" s="4"/>
+      <c r="BF21" s="4"/>
+      <c r="BG21" s="4"/>
+      <c r="BH21" s="4"/>
+      <c r="BI21" s="4"/>
+      <c r="BJ21" s="4"/>
+      <c r="BK21" s="4"/>
+      <c r="BL21" s="4"/>
+      <c r="BM21" s="4"/>
+      <c r="BN21" s="4"/>
+      <c r="BO21" s="4"/>
+      <c r="BP21" s="4"/>
+      <c r="BQ21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4"/>
+      <c r="A22" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="4"/>
+      <c r="Q22" s="4"/>
+      <c r="R22" s="4"/>
+      <c r="S22" s="4"/>
+      <c r="T22" s="4"/>
+      <c r="U22" s="4"/>
+      <c r="V22" s="4"/>
+      <c r="W22" s="4"/>
+      <c r="X22" s="4"/>
+      <c r="Y22" s="4"/>
+      <c r="Z22" s="4"/>
+      <c r="AA22" s="4"/>
+      <c r="AB22" s="4"/>
+      <c r="AC22" s="4"/>
+      <c r="AD22" s="4"/>
+      <c r="AE22" s="4"/>
+      <c r="AF22" s="4"/>
+      <c r="AG22" s="4"/>
+      <c r="AH22" s="4"/>
+      <c r="AI22" s="4"/>
+      <c r="AJ22" s="4"/>
+      <c r="AK22" s="4"/>
+      <c r="AL22" s="4"/>
+      <c r="AM22" s="4"/>
+      <c r="AN22" s="4"/>
+      <c r="AO22" s="4"/>
+      <c r="AP22" s="4"/>
+      <c r="AQ22" s="4"/>
+      <c r="AR22" s="4"/>
+      <c r="AS22" s="4"/>
+      <c r="AT22" s="4"/>
+      <c r="AU22" s="4"/>
+      <c r="AV22" s="4"/>
+      <c r="AW22" s="4"/>
+      <c r="AX22" s="4"/>
+      <c r="AY22" s="4"/>
+      <c r="AZ22" s="4"/>
+      <c r="BA22" s="4"/>
+      <c r="BB22" s="4"/>
+      <c r="BC22" s="4"/>
+      <c r="BD22" s="4"/>
+      <c r="BE22" s="4"/>
+      <c r="BF22" s="4"/>
+      <c r="BG22" s="4"/>
+      <c r="BH22" s="4"/>
+      <c r="BI22" s="4"/>
+      <c r="BJ22" s="4"/>
+      <c r="BK22" s="4"/>
+      <c r="BL22" s="4"/>
+      <c r="BM22" s="4"/>
+      <c r="BN22" s="4"/>
+      <c r="BO22" s="4"/>
+      <c r="BP22" s="4"/>
+      <c r="BQ22" s="4"/>
     </row>
-    <row r="23" customFormat="false" ht="14.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
-        <v>143</v>
-      </c>
-      <c r="B23" s="21"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="21"/>
-      <c r="I23" s="21"/>
-      <c r="J23" s="21"/>
-      <c r="K23" s="21"/>
-      <c r="L23" s="21"/>
-      <c r="M23" s="21"/>
-      <c r="N23" s="21"/>
-      <c r="O23" s="21"/>
-      <c r="P23" s="21"/>
-      <c r="Q23" s="21"/>
-      <c r="R23" s="21"/>
-      <c r="S23" s="21"/>
-      <c r="T23" s="21"/>
-      <c r="U23" s="21"/>
-      <c r="V23" s="21"/>
-      <c r="W23" s="21"/>
-      <c r="X23" s="21"/>
-      <c r="Y23" s="21"/>
-      <c r="Z23" s="21"/>
-      <c r="AA23" s="21"/>
-      <c r="AB23" s="21"/>
-      <c r="AC23" s="21"/>
-      <c r="AD23" s="21"/>
-      <c r="AE23" s="21"/>
-      <c r="AF23" s="21"/>
-      <c r="AG23" s="21"/>
-      <c r="AH23" s="21"/>
-      <c r="AI23" s="21"/>
-      <c r="AJ23" s="21"/>
-      <c r="AK23" s="21"/>
-      <c r="AL23" s="21"/>
-      <c r="AM23" s="21"/>
-      <c r="AN23" s="21"/>
-      <c r="AO23" s="21"/>
-      <c r="AP23" s="21"/>
-      <c r="AQ23" s="21"/>
-      <c r="AR23" s="21"/>
-      <c r="AS23" s="21"/>
-      <c r="AT23" s="21"/>
-      <c r="AU23" s="21"/>
-      <c r="AV23" s="21"/>
-      <c r="AW23" s="21"/>
-      <c r="AX23" s="21"/>
-      <c r="AY23" s="21"/>
-      <c r="AZ23" s="21"/>
-      <c r="BA23" s="21"/>
-      <c r="BB23" s="21"/>
-      <c r="BC23" s="21"/>
-      <c r="BD23" s="21"/>
-      <c r="BE23" s="21"/>
-      <c r="BF23" s="21"/>
-      <c r="BG23" s="21"/>
-      <c r="BH23" s="21"/>
-      <c r="BI23" s="21"/>
-      <c r="BJ23" s="21"/>
-      <c r="BK23" s="21"/>
-      <c r="BL23" s="21"/>
-      <c r="BM23" s="21"/>
-      <c r="BN23" s="21"/>
-      <c r="BO23" s="21"/>
-      <c r="BP23" s="21"/>
-      <c r="BQ23" s="21"/>
+    <row r="23" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4"/>
+      <c r="O23" s="4"/>
+      <c r="P23" s="4"/>
+      <c r="Q23" s="4"/>
+      <c r="R23" s="4"/>
+      <c r="S23" s="4"/>
+      <c r="T23" s="4"/>
+      <c r="U23" s="4"/>
+      <c r="V23" s="4"/>
+      <c r="W23" s="4"/>
+      <c r="X23" s="4"/>
+      <c r="Y23" s="4"/>
+      <c r="Z23" s="4"/>
+      <c r="AA23" s="4"/>
+      <c r="AB23" s="4"/>
+      <c r="AC23" s="4"/>
+      <c r="AD23" s="4"/>
+      <c r="AE23" s="4"/>
+      <c r="AF23" s="4"/>
+      <c r="AG23" s="4"/>
+      <c r="AH23" s="4"/>
+      <c r="AI23" s="4"/>
+      <c r="AJ23" s="4"/>
+      <c r="AK23" s="4"/>
+      <c r="AL23" s="4"/>
+      <c r="AM23" s="4"/>
+      <c r="AN23" s="4"/>
+      <c r="AO23" s="4"/>
+      <c r="AP23" s="4"/>
+      <c r="AQ23" s="4"/>
+      <c r="AR23" s="4"/>
+      <c r="AS23" s="4"/>
+      <c r="AT23" s="4"/>
+      <c r="AU23" s="4"/>
+      <c r="AV23" s="4"/>
+      <c r="AW23" s="4"/>
+      <c r="AX23" s="4"/>
+      <c r="AY23" s="4"/>
+      <c r="AZ23" s="4"/>
+      <c r="BA23" s="4"/>
+      <c r="BB23" s="4"/>
+      <c r="BC23" s="4"/>
+      <c r="BD23" s="4"/>
+      <c r="BE23" s="4"/>
+      <c r="BF23" s="4"/>
+      <c r="BG23" s="4"/>
+      <c r="BH23" s="4"/>
+      <c r="BI23" s="4"/>
+      <c r="BJ23" s="4"/>
+      <c r="BK23" s="4"/>
+      <c r="BL23" s="4"/>
+      <c r="BM23" s="4"/>
+      <c r="BN23" s="4"/>
+      <c r="BO23" s="4"/>
+      <c r="BP23" s="4"/>
+      <c r="BQ23" s="4"/>
     </row>
     <row r="24" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>79</v>
+        <v>129</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -20255,7 +19814,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>144</v>
+        <v>26</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -20328,7 +19887,7 @@
     </row>
     <row r="26" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -20401,7 +19960,7 @@
     </row>
     <row r="27" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -20474,7 +20033,7 @@
     </row>
     <row r="28" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>26</v>
+        <v>132</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -20547,7 +20106,7 @@
     </row>
     <row r="29" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -20620,7 +20179,7 @@
     </row>
     <row r="30" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -20691,227 +20250,8 @@
       <c r="BP30" s="4"/>
       <c r="BQ30" s="4"/>
     </row>
-    <row r="31" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
-      <c r="I31" s="4"/>
-      <c r="J31" s="4"/>
-      <c r="K31" s="4"/>
-      <c r="L31" s="4"/>
-      <c r="M31" s="4"/>
-      <c r="N31" s="4"/>
-      <c r="O31" s="4"/>
-      <c r="P31" s="4"/>
-      <c r="Q31" s="4"/>
-      <c r="R31" s="4"/>
-      <c r="S31" s="4"/>
-      <c r="T31" s="4"/>
-      <c r="U31" s="4"/>
-      <c r="V31" s="4"/>
-      <c r="W31" s="4"/>
-      <c r="X31" s="4"/>
-      <c r="Y31" s="4"/>
-      <c r="Z31" s="4"/>
-      <c r="AA31" s="4"/>
-      <c r="AB31" s="4"/>
-      <c r="AC31" s="4"/>
-      <c r="AD31" s="4"/>
-      <c r="AE31" s="4"/>
-      <c r="AF31" s="4"/>
-      <c r="AG31" s="4"/>
-      <c r="AH31" s="4"/>
-      <c r="AI31" s="4"/>
-      <c r="AJ31" s="4"/>
-      <c r="AK31" s="4"/>
-      <c r="AL31" s="4"/>
-      <c r="AM31" s="4"/>
-      <c r="AN31" s="4"/>
-      <c r="AO31" s="4"/>
-      <c r="AP31" s="4"/>
-      <c r="AQ31" s="4"/>
-      <c r="AR31" s="4"/>
-      <c r="AS31" s="4"/>
-      <c r="AT31" s="4"/>
-      <c r="AU31" s="4"/>
-      <c r="AV31" s="4"/>
-      <c r="AW31" s="4"/>
-      <c r="AX31" s="4"/>
-      <c r="AY31" s="4"/>
-      <c r="AZ31" s="4"/>
-      <c r="BA31" s="4"/>
-      <c r="BB31" s="4"/>
-      <c r="BC31" s="4"/>
-      <c r="BD31" s="4"/>
-      <c r="BE31" s="4"/>
-      <c r="BF31" s="4"/>
-      <c r="BG31" s="4"/>
-      <c r="BH31" s="4"/>
-      <c r="BI31" s="4"/>
-      <c r="BJ31" s="4"/>
-      <c r="BK31" s="4"/>
-      <c r="BL31" s="4"/>
-      <c r="BM31" s="4"/>
-      <c r="BN31" s="4"/>
-      <c r="BO31" s="4"/>
-      <c r="BP31" s="4"/>
-      <c r="BQ31" s="4"/>
-    </row>
-    <row r="32" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
-      <c r="I32" s="4"/>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
-      <c r="L32" s="4"/>
-      <c r="M32" s="4"/>
-      <c r="N32" s="4"/>
-      <c r="O32" s="4"/>
-      <c r="P32" s="4"/>
-      <c r="Q32" s="4"/>
-      <c r="R32" s="4"/>
-      <c r="S32" s="4"/>
-      <c r="T32" s="4"/>
-      <c r="U32" s="4"/>
-      <c r="V32" s="4"/>
-      <c r="W32" s="4"/>
-      <c r="X32" s="4"/>
-      <c r="Y32" s="4"/>
-      <c r="Z32" s="4"/>
-      <c r="AA32" s="4"/>
-      <c r="AB32" s="4"/>
-      <c r="AC32" s="4"/>
-      <c r="AD32" s="4"/>
-      <c r="AE32" s="4"/>
-      <c r="AF32" s="4"/>
-      <c r="AG32" s="4"/>
-      <c r="AH32" s="4"/>
-      <c r="AI32" s="4"/>
-      <c r="AJ32" s="4"/>
-      <c r="AK32" s="4"/>
-      <c r="AL32" s="4"/>
-      <c r="AM32" s="4"/>
-      <c r="AN32" s="4"/>
-      <c r="AO32" s="4"/>
-      <c r="AP32" s="4"/>
-      <c r="AQ32" s="4"/>
-      <c r="AR32" s="4"/>
-      <c r="AS32" s="4"/>
-      <c r="AT32" s="4"/>
-      <c r="AU32" s="4"/>
-      <c r="AV32" s="4"/>
-      <c r="AW32" s="4"/>
-      <c r="AX32" s="4"/>
-      <c r="AY32" s="4"/>
-      <c r="AZ32" s="4"/>
-      <c r="BA32" s="4"/>
-      <c r="BB32" s="4"/>
-      <c r="BC32" s="4"/>
-      <c r="BD32" s="4"/>
-      <c r="BE32" s="4"/>
-      <c r="BF32" s="4"/>
-      <c r="BG32" s="4"/>
-      <c r="BH32" s="4"/>
-      <c r="BI32" s="4"/>
-      <c r="BJ32" s="4"/>
-      <c r="BK32" s="4"/>
-      <c r="BL32" s="4"/>
-      <c r="BM32" s="4"/>
-      <c r="BN32" s="4"/>
-      <c r="BO32" s="4"/>
-      <c r="BP32" s="4"/>
-      <c r="BQ32" s="4"/>
-    </row>
-    <row r="33" customFormat="false" ht="12.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
-      <c r="L33" s="4"/>
-      <c r="M33" s="4"/>
-      <c r="N33" s="4"/>
-      <c r="O33" s="4"/>
-      <c r="P33" s="4"/>
-      <c r="Q33" s="4"/>
-      <c r="R33" s="4"/>
-      <c r="S33" s="4"/>
-      <c r="T33" s="4"/>
-      <c r="U33" s="4"/>
-      <c r="V33" s="4"/>
-      <c r="W33" s="4"/>
-      <c r="X33" s="4"/>
-      <c r="Y33" s="4"/>
-      <c r="Z33" s="4"/>
-      <c r="AA33" s="4"/>
-      <c r="AB33" s="4"/>
-      <c r="AC33" s="4"/>
-      <c r="AD33" s="4"/>
-      <c r="AE33" s="4"/>
-      <c r="AF33" s="4"/>
-      <c r="AG33" s="4"/>
-      <c r="AH33" s="4"/>
-      <c r="AI33" s="4"/>
-      <c r="AJ33" s="4"/>
-      <c r="AK33" s="4"/>
-      <c r="AL33" s="4"/>
-      <c r="AM33" s="4"/>
-      <c r="AN33" s="4"/>
-      <c r="AO33" s="4"/>
-      <c r="AP33" s="4"/>
-      <c r="AQ33" s="4"/>
-      <c r="AR33" s="4"/>
-      <c r="AS33" s="4"/>
-      <c r="AT33" s="4"/>
-      <c r="AU33" s="4"/>
-      <c r="AV33" s="4"/>
-      <c r="AW33" s="4"/>
-      <c r="AX33" s="4"/>
-      <c r="AY33" s="4"/>
-      <c r="AZ33" s="4"/>
-      <c r="BA33" s="4"/>
-      <c r="BB33" s="4"/>
-      <c r="BC33" s="4"/>
-      <c r="BD33" s="4"/>
-      <c r="BE33" s="4"/>
-      <c r="BF33" s="4"/>
-      <c r="BG33" s="4"/>
-      <c r="BH33" s="4"/>
-      <c r="BI33" s="4"/>
-      <c r="BJ33" s="4"/>
-      <c r="BK33" s="4"/>
-      <c r="BL33" s="4"/>
-      <c r="BM33" s="4"/>
-      <c r="BN33" s="4"/>
-      <c r="BO33" s="4"/>
-      <c r="BP33" s="4"/>
-      <c r="BQ33" s="4"/>
-    </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="24">
     <mergeCell ref="A1:BM1"/>
     <mergeCell ref="BN1:BQ1"/>
     <mergeCell ref="A2:BQ2"/>
@@ -20924,10 +20264,10 @@
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="B11:E11"/>
     <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B14:E14"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="A17:Z17"/>
+    <mergeCell ref="A14:Z14"/>
+    <mergeCell ref="A20:BQ20"/>
+    <mergeCell ref="A21:BQ21"/>
+    <mergeCell ref="A22:BQ22"/>
     <mergeCell ref="A23:BQ23"/>
     <mergeCell ref="A24:BQ24"/>
     <mergeCell ref="A25:BQ25"/>
@@ -20936,9 +20276,6 @@
     <mergeCell ref="A28:BQ28"/>
     <mergeCell ref="A29:BQ29"/>
     <mergeCell ref="A30:BQ30"/>
-    <mergeCell ref="A31:BQ31"/>
-    <mergeCell ref="A32:BQ32"/>
-    <mergeCell ref="A33:BQ33"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>

</xml_diff>